<commit_message>
Dashboard builder: footnotes, chart-linked table actuals, current month
- Footnotes tab: per-month notes on one chart or all charts, shown as a
  superscript on the month label and listed under the charts.
- Table rows can take Month Actual and YTD Actual from the Charts tab
  (From Chart / From Component, YTD Method Sum or Average).
- Table headers renamed to Month EV Case / YTD EV Case; the old
  Comparison headers still load.
- Settings gains Current month, which drives the YTD window, the default
  month and YTD headings, and hides current-year bars after that month.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -8,9 +8,10 @@
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
     <sheet name="Settings" sheetId="2" r:id="rId2"/>
     <sheet name="Charts" sheetId="3" r:id="rId3"/>
-    <sheet name="Table" sheetId="4" r:id="rId4"/>
-    <sheet name="Commentary" sheetId="5" r:id="rId5"/>
-    <sheet name="Side Table" sheetId="6" r:id="rId6"/>
+    <sheet name="Footnotes" sheetId="4" r:id="rId4"/>
+    <sheet name="Table" sheetId="5" r:id="rId5"/>
+    <sheet name="Commentary" sheetId="6" r:id="rId6"/>
+    <sheet name="Side Table" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -156,7 +157,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="130" customWidth="1"/>
+    <col min="1" max="1" width="140" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -177,7 +178,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.  Fill in the Settings, Charts, Table, Commentary and Side Table tabs.  Blue text on yellow = inputs.</t>
+          <t xml:space="preserve">1.  Fill in the Settings, Charts, Footnotes, Table, Commentary and Side Table tabs.  Blue text on yellow = inputs.</t>
         </is>
       </c>
     </row>
@@ -191,7 +192,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.  Open "Dashboard Builder.html" in Edge or Chrome and drag this workbook onto the page.</t>
+          <t xml:space="preserve">3.  Open the Dashboard Builder page in Edge or Chrome and drag this workbook onto it.</t>
         </is>
       </c>
     </row>
@@ -220,69 +221,125 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charts  -  one row per chart / component / year with Jan-Dec values.  Leave months blank where there is no data yet.</t>
+          <t xml:space="preserve">               "Current month" drives the month and YTD columns of the table.  Current-year chart values after it are not shown.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Each distinct "Chart" name becomes its own chart.  Rows with a "Component" (e.g. Contracted, Merchant) are stacked.</t>
+          <t xml:space="preserve">Charts  -  one row per chart / component / year with Jan-Dec values.  Leave months blank where there is no data yet.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Every chart shows the Current year and Prior year from Settings side by side, month by month.</t>
+          <t xml:space="preserve">               Each distinct "Chart" name becomes its own chart.  Rows with a "Component" (e.g. Contracted, Merchant) are stacked.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Table  -  any number of rows.  The variance is calculated for you; "Better When" sets whether it shows green or red.</t>
+          <t xml:space="preserve">               Every chart shows the Prior year and Current year from Settings side by side, month by month.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
+          <t xml:space="preserve">               Enter full precision here (e.g. 3.92); the Decimals column only controls how the chart labels are rounded.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+          <t xml:space="preserve">Footnotes  -  explain a month on a chart.  Leave "Chart" blank to mark that month on every chart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               The month label gets a small number and the note prints under the charts.</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tips</t>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Table  -  any number of rows.  The variance is calculated for you; "Better When" sets whether it shows green or red.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
+          <t xml:space="preserve">               Put a chart name in "From Chart" to fill Month Actual and YTD Actual from the Charts tab automatically</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+          <t xml:space="preserve">               (add a "From Component" to use just one component, e.g. Contracted).  Leave "From Chart" blank to type the actuals yourself.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tips</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -299,7 +356,7 @@
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="70" customWidth="1"/>
-    <col min="3" max="3" width="70" customWidth="1"/>
+    <col min="3" max="3" width="90" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,271 +477,283 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chart section title</t>
+          <t xml:space="preserve">Current month</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Monthly Performance - 2026 vs. 2025</t>
+          <t xml:space="preserve">Aug</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header above the charts.</t>
+          <t xml:space="preserve">The month being reported.  Drives Month Actual and YTD (Jan through this month) in the table.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data labels</t>
+          <t xml:space="preserve">Chart section title</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">This year</t>
+          <t xml:space="preserve">Monthly Performance - 2026 vs. 2025</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which bars get value labels: This year / Both years / None.</t>
+          <t xml:space="preserve">Header above the charts.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chart columns</t>
+          <t xml:space="preserve">Data labels</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto</t>
+          <t xml:space="preserve">This year</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto = 1 column for up to 3 charts, 2 columns for more.</t>
+          <t xml:space="preserve">Which bars get value labels: This year / Both years / None.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Table title</t>
+          <t xml:space="preserve">Chart columns</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operating and Financial Performance vs. Budget - Monthly &amp; YTD</t>
+          <t xml:space="preserve">Auto</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header above the comparison table.</t>
+          <t xml:space="preserve">Auto = 1 column for up to 3 charts, 2 columns for more.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Month heading</t>
+          <t xml:space="preserve">Table title</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">August</t>
+          <t xml:space="preserve">Operating and Financial Performance vs. EV Case - Monthly &amp; YTD</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heading over the monthly columns, e.g. August.</t>
+          <t xml:space="preserve">Header above the comparison table.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">YTD heading</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YTD Through August</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Month heading</t>
+        </is>
+      </c>
+      <c r="B13" s="8"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heading over the year-to-date columns.</t>
+          <t xml:space="preserve">Heading over the monthly columns.  Leave blank to use the Current month (e.g. August).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Actual label</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Actual</t>
-        </is>
-      </c>
+          <t xml:space="preserve">YTD heading</t>
+        </is>
+      </c>
+      <c r="B14" s="8"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Column label for actual values.</t>
+          <t xml:space="preserve">Heading over the year-to-date columns.  Leave blank for "YTD Through August".</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparison label</t>
+          <t xml:space="preserve">Actual label</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Budget</t>
+          <t xml:space="preserve">Actual</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Column label for the comparison case (EV Case, Budget, Forecast...).</t>
+          <t xml:space="preserve">Column label for actual values.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variance label</t>
+          <t xml:space="preserve">Comparison label</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Variance</t>
+          <t xml:space="preserve">EV Case</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Column label for the variance.</t>
+          <t xml:space="preserve">Column label for the comparison case (EV Case, Budget, Forecast...).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Negative numbers</t>
+          <t xml:space="preserve">Variance label</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parentheses</t>
+          <t xml:space="preserve">Variance</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parentheses: (1.8)   Minus sign: -1.8</t>
+          <t xml:space="preserve">Column label for the variance.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side panel type</t>
+          <t xml:space="preserve">Negative numbers</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commentary</t>
+          <t xml:space="preserve">Parentheses</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commentary / Table / Table + Commentary / None.</t>
+          <t xml:space="preserve">Parentheses: (1.8)   Minus sign: -1.8</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side panel title</t>
+          <t xml:space="preserve">Side panel type</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maintenance Commentary</t>
+          <t xml:space="preserve">Commentary</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header of the bottom-right box.</t>
+          <t xml:space="preserve">Commentary / Table / Table + Commentary / None.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side panel width %</t>
-        </is>
-      </c>
-      <c r="B20" s="8">
-        <v>30</v>
+          <t xml:space="preserve">Side panel title</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maintenance Commentary</t>
+        </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Width of the bottom-right box as a share of the page (15-50).</t>
+          <t xml:space="preserve">Header of the bottom-right box.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Footer</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sources: Bluefield monthly operating reports; 2026 budget model.  Fictional example data.</t>
-        </is>
+          <t xml:space="preserve">Side panel width %</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <v>30</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources line at the bottom of the page.</t>
+          <t xml:space="preserve">Width of the bottom-right box as a share of the page (15-50).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Footer</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sources: Bluefield monthly operating reports; 2026 EV Case model.  Fictional example data.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sources line at the bottom of the page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Page size</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Letter</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Letter or A4 (always landscape).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+      <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10">
       <formula1>"This year,Both years,None"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11">
       <formula1>"Auto,1,2,3"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B18">
       <formula1>"Parentheses,Minus sign"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B19">
       <formula1>"Commentary,Table,Table + Commentary,None"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B22">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23">
       <formula1>"Letter,A4"</formula1>
     </dataValidation>
   </dataValidations>
@@ -828,7 +897,7 @@
         <v>52.4</v>
       </c>
       <c r="K2" s="9">
-        <v>51.7</v>
+        <v>41.7</v>
       </c>
       <c r="L2" s="9">
         <v>47.2</v>
@@ -901,34 +970,34 @@
       <c r="D4" s="8">
         <v>1</v>
       </c>
-      <c r="E4" s="9">
-        <v>1.6</v>
-      </c>
-      <c r="F4" s="9">
-        <v>1.8</v>
-      </c>
-      <c r="G4" s="9">
-        <v>2.6</v>
-      </c>
-      <c r="H4" s="9">
-        <v>3</v>
-      </c>
-      <c r="I4" s="9">
-        <v>3.4</v>
-      </c>
-      <c r="J4" s="9">
-        <v>4.1</v>
-      </c>
-      <c r="K4" s="9">
-        <v>4.3</v>
-      </c>
-      <c r="L4" s="9">
-        <v>3.9</v>
-      </c>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
+      <c r="E4" s="10">
+        <v>1.62</v>
+      </c>
+      <c r="F4" s="10">
+        <v>1.84</v>
+      </c>
+      <c r="G4" s="10">
+        <v>2.57</v>
+      </c>
+      <c r="H4" s="10">
+        <v>3.03</v>
+      </c>
+      <c r="I4" s="10">
+        <v>3.41</v>
+      </c>
+      <c r="J4" s="10">
+        <v>4.12</v>
+      </c>
+      <c r="K4" s="10">
+        <v>3.46</v>
+      </c>
+      <c r="L4" s="10">
+        <v>3.92</v>
+      </c>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -993,34 +1062,34 @@
       <c r="D6" s="8">
         <v>1</v>
       </c>
-      <c r="E6" s="9">
-        <v>-0.4</v>
-      </c>
-      <c r="F6" s="9">
-        <v>0.1</v>
-      </c>
-      <c r="G6" s="9">
-        <v>0.9</v>
-      </c>
-      <c r="H6" s="9">
-        <v>1.3</v>
-      </c>
-      <c r="I6" s="9">
-        <v>1.7</v>
-      </c>
-      <c r="J6" s="9">
-        <v>2.3</v>
-      </c>
-      <c r="K6" s="9">
-        <v>2.5</v>
-      </c>
-      <c r="L6" s="9">
-        <v>2.1</v>
-      </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
+      <c r="E6" s="10">
+        <v>-0.41</v>
+      </c>
+      <c r="F6" s="10">
+        <v>0.12</v>
+      </c>
+      <c r="G6" s="10">
+        <v>0.88</v>
+      </c>
+      <c r="H6" s="10">
+        <v>1.31</v>
+      </c>
+      <c r="I6" s="10">
+        <v>1.69</v>
+      </c>
+      <c r="J6" s="10">
+        <v>2.27</v>
+      </c>
+      <c r="K6" s="10">
+        <v>1.66</v>
+      </c>
+      <c r="L6" s="10">
+        <v>2.07</v>
+      </c>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1081,246 +1150,77 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="100" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Metric</t>
+          <t xml:space="preserve">Chart</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prefix</t>
+          <t xml:space="preserve">Month</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suffix</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decimals</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Better When</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Variance As</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bold</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Month Actual</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Month Comparison</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YTD Actual</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YTD Comparison</t>
+          <t xml:space="preserve">Note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generation</t>
-        </is>
-      </c>
-      <c r="B2" s="8"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jul</t>
+        </is>
+      </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GWh</t>
-        </is>
-      </c>
-      <c r="D2" s="8">
-        <v>1</v>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Higher</t>
-        </is>
-      </c>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="9">
-        <v>47.2</v>
-      </c>
-      <c r="I2" s="9">
-        <v>50.6</v>
-      </c>
-      <c r="J2" s="9">
-        <v>336</v>
-      </c>
-      <c r="K2" s="9">
-        <v>351.4</v>
+          <t xml:space="preserve">Plant shut down July 13-17 for a utility transformer replacement at the point of interconnection.</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Revenue</t>
+          <t xml:space="preserve">Operating income ($MM)</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">$</t>
+          <t xml:space="preserve">Jan</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">MM</t>
-        </is>
-      </c>
-      <c r="D3" s="8">
-        <v>2</v>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Higher</t>
-        </is>
-      </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="10">
-        <v>3.92</v>
-      </c>
-      <c r="I3" s="10">
-        <v>3.85</v>
-      </c>
-      <c r="J3" s="10">
-        <v>24.71</v>
-      </c>
-      <c r="K3" s="10">
-        <v>25.3</v>
+          <t xml:space="preserve">Annual property insurance premium expensed in January.</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">O&amp;M expense</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MM</t>
-        </is>
-      </c>
-      <c r="D4" s="8">
-        <v>2</v>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lower</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Abs</t>
-        </is>
-      </c>
-      <c r="G4" s="8"/>
-      <c r="H4" s="10">
-        <v>0.86</v>
-      </c>
-      <c r="I4" s="10">
-        <v>0.74</v>
-      </c>
-      <c r="J4" s="10">
-        <v>6.12</v>
-      </c>
-      <c r="K4" s="10">
-        <v>6.4</v>
-      </c>
+      <c r="A4" s="8"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Operating income</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MM</t>
-        </is>
-      </c>
-      <c r="D5" s="8">
-        <v>2</v>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Higher</t>
-        </is>
-      </c>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Y</t>
-        </is>
-      </c>
-      <c r="H5" s="10">
-        <v>2.07</v>
-      </c>
-      <c r="I5" s="10">
-        <v>2.31</v>
-      </c>
-      <c r="J5" s="10">
-        <v>10.48</v>
-      </c>
-      <c r="K5" s="10">
-        <v>11.62</v>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E200">
-      <formula1>"Higher,Lower"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F200">
-      <formula1>"%,Abs,Pts"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G200">
-      <formula1>"Y,N"</formula1>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B200">
+      <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1331,6 +1231,329 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="7" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From Chart</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">From Component</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YTD Method</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prefix</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suffix</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decimals</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Better When</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Variance As</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bold</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Month Actual</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Month EV Case</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YTD Actual</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YTD EV Case</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generation</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generation (GWh)</t>
+        </is>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> GWh</t>
+        </is>
+      </c>
+      <c r="G2" s="8">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Higher</t>
+        </is>
+      </c>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(from Charts)</t>
+        </is>
+      </c>
+      <c r="L2" s="9">
+        <v>50.6</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(from Charts)</t>
+        </is>
+      </c>
+      <c r="N2" s="9">
+        <v>351.4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revenue</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revenue ($MM)</t>
+        </is>
+      </c>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MM</t>
+        </is>
+      </c>
+      <c r="G3" s="8">
+        <v>2</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Higher</t>
+        </is>
+      </c>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(from Charts)</t>
+        </is>
+      </c>
+      <c r="L3" s="10">
+        <v>3.85</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(from Charts)</t>
+        </is>
+      </c>
+      <c r="N3" s="10">
+        <v>25.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O&amp;M expense</t>
+        </is>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MM</t>
+        </is>
+      </c>
+      <c r="G4" s="8">
+        <v>2</v>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abs</t>
+        </is>
+      </c>
+      <c r="J4" s="8"/>
+      <c r="K4" s="10">
+        <v>0.86</v>
+      </c>
+      <c r="L4" s="10">
+        <v>0.74</v>
+      </c>
+      <c r="M4" s="10">
+        <v>6.12</v>
+      </c>
+      <c r="N4" s="10">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operating income</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operating income ($MM)</t>
+        </is>
+      </c>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MM</t>
+        </is>
+      </c>
+      <c r="G5" s="8">
+        <v>2</v>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Higher</t>
+        </is>
+      </c>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(from Charts)</t>
+        </is>
+      </c>
+      <c r="L5" s="10">
+        <v>2.31</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(from Charts)</t>
+        </is>
+      </c>
+      <c r="N5" s="10">
+        <v>11.62</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D200">
+      <formula1>"Sum,Average"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H200">
+      <formula1>"Higher,Lower"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I200">
+      <formula1>"%,Abs,Pts"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J200">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
@@ -1350,12 +1573,12 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Inverter block 3</t>
+          <t xml:space="preserve">Interconnection</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two central inverters offline August 4-9 for warranty replacement of power modules.</t>
+          <t xml:space="preserve">Utility replaced the POI transformer July 13-17; the plant was offline for the full outage.</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Dashboard builder: label prior-year bars too by default
Data labels now default to Both years, prior-year bars included (stacked
segments as well), in a slightly lighter ink than the current year.  The
example workbooks use the new default.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -516,12 +516,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">This year</t>
+          <t xml:space="preserve">Both years</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which bars get value labels: This year / Both years / None.</t>
+          <t xml:space="preserve">Which bars get value labels: Both years / This year / None.</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10">
-      <formula1>"This year,Both years,None"</formula1>
+      <formula1>"Both years,This year,None"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B11">
       <formula1>"Auto,1,2,3"</formula1>

</xml_diff>

<commit_message>
Dashboard builder: chart-name dropdowns in the example workbooks
Footnotes > Chart and Table > From Chart now offer a dropdown of the
distinct chart names on the Charts tab.  A hidden Lists tab derives the
names with a non-array unique-list formula (works in every Excel
version), exposed through a dynamic ChartNames defined name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -12,7 +12,12 @@
     <sheet name="Table" sheetId="5" r:id="rId5"/>
     <sheet name="Commentary" sheetId="6" r:id="rId6"/>
     <sheet name="Side Table" sheetId="7" r:id="rId7"/>
+    <sheet name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
   </sheets>
+  <definedNames>
+    <definedName name="ChartNames">OFFSET(Lists!$A$2,0,0,MAX(1,COUNTIF(Lists!$A$2:$A$101,"?*")),1)</definedName>
+  </definedNames>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -256,7 +261,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Footnotes  -  explain a month on a chart.  Leave "Chart" blank to mark that month on every chart.</t>
+          <t xml:space="preserve">Footnotes  -  explain a month on a chart.  Pick the chart from the dropdown, or leave "Chart" blank to mark that month on every chart.</t>
         </is>
       </c>
     </row>
@@ -277,7 +282,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Put a chart name in "From Chart" to fill Month Actual and YTD Actual from the Charts tab automatically</t>
+          <t xml:space="preserve">               Pick a chart in "From Chart" (dropdown) to fill Month Actual and YTD Actual from the Charts tab automatically</t>
         </is>
       </c>
     </row>
@@ -340,6 +345,13 @@
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -1218,7 +1230,10 @@
       <c r="C6" s="8"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A200">
+      <formula1>ChartNames</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B200">
       <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
@@ -1532,7 +1547,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B200">
+      <formula1>ChartNames</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D200">
       <formula1>"Sum,Average"</formula1>
     </dataValidation>
@@ -1637,4 +1655,623 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chart names</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A1,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A2,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A3,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A4,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A5,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A6,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A7,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A8,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A9,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A10,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A11,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A12,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A13,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A14,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A15,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A16,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A17,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A18,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A19,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A20,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A21,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A22,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A23,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A24,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A25,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A26,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A27,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A28,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A29,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A30,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A31,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A32,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A33,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A34,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A35,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A36,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A37,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A38,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A39,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A40,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A41,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A42,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A43,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A44,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A45,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A46,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A47,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A48,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A49,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A50,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A51,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A52,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A53,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A54,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A55,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A56,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A57,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A58,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A59,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A60,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A61,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A62,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A63,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A64,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A65,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A66,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A67,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A68,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A69,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A70,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A71,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A72,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A73,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A74,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A75,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A76,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A77,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A78,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A79,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A80,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A81,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A82,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A83,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A84,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A85,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A86,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A87,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A88,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A89,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A90,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A91,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A92,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A93,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A94,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A95,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A96,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A97,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A98,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A99,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A100,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard builder: optional page 2 for LTM debt service coverage
A Debt Service tab (quarterly Revenue / Expense / Debt service rows) adds
a second page: CFADS vs. stacked debt service by quarter, quarterly DSCR
bars with the LTM DSCR line and lock-up / default covenant lines, and a
cash flow table (revenue less expenses = CFADS, principal + interest =
debt service, quarterly and LTM DSCR) with an LTM column.  New settings
control inclusion, quarters shown, covenant levels, units and decimals.
The page container now holds one or two pages for screen and print.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -12,7 +12,9 @@
     <sheet name="Table" sheetId="5" r:id="rId5"/>
     <sheet name="Commentary" sheetId="6" r:id="rId6"/>
     <sheet name="Side Table" sheetId="7" r:id="rId7"/>
-    <sheet name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="Debt Service" sheetId="8" r:id="rId8"/>
+    <sheet name="DSCR Notes" sheetId="9" r:id="rId9"/>
+    <sheet name="Lists" sheetId="10" state="hidden" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="ChartNames">OFFSET(Lists!$A$2,0,0,MAX(1,COUNTIF(Lists!$A$2:$A$101,"?*")),1)</definedName>
@@ -321,40 +323,687 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt Service  -  quarterly cash flow for page 2.  One column per quarter, oldest on the left.  Role: Revenue, Expense or Debt service.</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tips</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  CFADS = Revenue - Expenses.  DSCR = CFADS / Debt service.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
+          <t xml:space="preserve">               LTM DSCR = last 4 quarters of CFADS / last 4 quarters of debt service.  Add any expense or debt service rows you need.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown beside the cash flow table on page 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tips</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chart names</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A1,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A2,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A3,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A4,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A5,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A6,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A7,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A8,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A9,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A10,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A11,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A12,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A13,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A14,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A15,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A16,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A17,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A18,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A19,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A20,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A21,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A22,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A23,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A24,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A25,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A26,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A27,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
-        </is>
+      <c r="A29" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A28,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
-        </is>
+      <c r="A30" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A29,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A30,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A31,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A32,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A33,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A34,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A35,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A36,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A37,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A38,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A39,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A40,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A41,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A42,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A43,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A44,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A45,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A46,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A47,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A48,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A49,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A50,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A51,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A52,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A53,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A54,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A55,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A56,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A57,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A58,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A59,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A60,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A61,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A62,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A63,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A64,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A65,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A66,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A67,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A68,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A69,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A70,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A71,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A72,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A73,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A74,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A75,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A76,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A77,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A78,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A79,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A80,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A81,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A82,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A83,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A84,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A85,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A86,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A87,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A88,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A89,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A90,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A91,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A92,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A93,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A94,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A95,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A96,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A97,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A98,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A99,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A100,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -748,8 +1397,119 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Include DSCR page</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto = add page 2 (Debt Service Coverage) when the Debt Service tab has data.  Yes / No to force it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DSCR page title</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt Service Coverage - LTM Basis</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header above the DSCR charts on page 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quarters shown</t>
+        </is>
+      </c>
+      <c r="B26" s="8">
+        <v>4</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How many of the most recent quarters page 2 shows (1-8).  Enter 3 extra older quarters to show an LTM DSCR for every quarter shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lock-up DSCR</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Distribution lock-up covenant, e.g. 1.20.  Drawn as a reference line; leave blank for none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Default DSCR</t>
+        </is>
+      </c>
+      <c r="B28" s="8">
+        <v>1.1</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Default covenant, e.g. 1.10.  Drawn as a reference line; leave blank for none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cash flow units</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$MM</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units label for page 2, e.g. $MM or $000s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cash flow decimals</t>
+        </is>
+      </c>
+      <c r="B30" s="8">
+        <v>2</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decimals in the page 2 cash flow table.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
       <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
@@ -767,6 +1527,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23">
       <formula1>"Letter,A4"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B24">
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1661,614 +2424,336 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chart names</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Role</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4 2024</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q1 2025</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q2 2025</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 2025</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4 2025</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q1 2026</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q2 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A1,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revenue</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revenue</t>
+        </is>
+      </c>
+      <c r="C2" s="10">
+        <v>5.31</v>
+      </c>
+      <c r="D2" s="10">
+        <v>5.62</v>
+      </c>
+      <c r="E2" s="10">
+        <v>10.04</v>
+      </c>
+      <c r="F2" s="10">
+        <v>10.52</v>
+      </c>
+      <c r="G2" s="10">
+        <v>5.93</v>
+      </c>
+      <c r="H2" s="10">
+        <v>6.08</v>
+      </c>
+      <c r="I2" s="10">
+        <v>10.61</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A2,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O&amp;M</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expense</t>
+        </is>
+      </c>
+      <c r="C3" s="10">
+        <v>1.92</v>
+      </c>
+      <c r="D3" s="10">
+        <v>2.01</v>
+      </c>
+      <c r="E3" s="10">
+        <v>2.08</v>
+      </c>
+      <c r="F3" s="10">
+        <v>2.17</v>
+      </c>
+      <c r="G3" s="10">
+        <v>2.03</v>
+      </c>
+      <c r="H3" s="10">
+        <v>2.11</v>
+      </c>
+      <c r="I3" s="10">
+        <v>2.19</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A3,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Property taxes</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expense</t>
+        </is>
+      </c>
+      <c r="C4" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="D4" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="E4" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="F4" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="G4" s="10">
+        <v>0.42</v>
+      </c>
+      <c r="H4" s="10">
+        <v>0.45</v>
+      </c>
+      <c r="I4" s="10">
+        <v>0.45</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A4,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Other taxes</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expense</t>
+        </is>
+      </c>
+      <c r="C5" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="D5" s="10">
+        <v>0.09</v>
+      </c>
+      <c r="E5" s="10">
+        <v>0.18</v>
+      </c>
+      <c r="F5" s="10">
+        <v>0.21</v>
+      </c>
+      <c r="G5" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="H5" s="10">
+        <v>0.08</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0.19</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A5,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Principal</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service</t>
+        </is>
+      </c>
+      <c r="C6" s="10">
+        <v>2.4</v>
+      </c>
+      <c r="D6" s="10">
+        <v>2.42</v>
+      </c>
+      <c r="E6" s="10">
+        <v>2.48</v>
+      </c>
+      <c r="F6" s="10">
+        <v>2.51</v>
+      </c>
+      <c r="G6" s="10">
+        <v>2.57</v>
+      </c>
+      <c r="H6" s="10">
+        <v>2.62</v>
+      </c>
+      <c r="I6" s="10">
+        <v>2.68</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A6,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interest</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service</t>
+        </is>
+      </c>
+      <c r="C7" s="10">
+        <v>1.91</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1.86</v>
+      </c>
+      <c r="E7" s="10">
+        <v>1.81</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1.76</v>
+      </c>
+      <c r="G7" s="10">
+        <v>1.7</v>
+      </c>
+      <c r="H7" s="10">
+        <v>1.65</v>
+      </c>
+      <c r="I7" s="10">
+        <v>1.6</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A7,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A8,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A9,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A10,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A11,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A12,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A13,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A14,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A15,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A16,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A17,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A18,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A19,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A20,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A21,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A22,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A23,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A24,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A25,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A26,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A27,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A28,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A29,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A30,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A31,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A32,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A33,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A34,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A35,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A36,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A37,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A38,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A39,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A40,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A41,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A42,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A43,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A44,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A45,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A46,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A47,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A48,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A49,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A50,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A51,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A52,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A53,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A54,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A55,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A56,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A57,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A58,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A59,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A60,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A61,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A62,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A63,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A64,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A65,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A66,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A67,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A68,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A69,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A70,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A71,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A72,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A73,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A74,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A75,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A76,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A77,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A78,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A79,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A80,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A81,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A82,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A83,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A84,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A85,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A86,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A87,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A88,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A89,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A90,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A91,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A92,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A93,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A94,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A95,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A96,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A97,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A98,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A99,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <f>IFERROR(INDEX(Charts!$A$2:$A$500,MATCH(0,INDEX(COUNTIF($A$1:A100,Charts!$A$2:$A$500)+(Charts!$A$2:$A$500=""),0),0)),"")</f>
-        <v/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B100">
+      <formula1>"Revenue,Expense,Debt service"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="90" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heading</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seasonality</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q1 and Q4 coverage falls below 1.0x on a stand-alone basis every year; the covenants test on an LTM basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Next test</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 2026 test at September 30, 2026.  Distributions require 1.20x LTM.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard builder: distribution lock-up naming, optional covenants, reserves
- Setting renamed to Distribution lock-up DSCR (the old Lock-up DSCR name
  still loads); labels on page 2 follow.
- A blank distribution lock-up or default DSCR leaves no trace: no
  reference line, legend entry, header text, or table coloring.
- New Reserves tab (required balance, balance available) renders below
  the DSCR chart with % funded and an underfunded flag, above any DSCR
  notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -13,8 +13,9 @@
     <sheet name="Commentary" sheetId="6" r:id="rId6"/>
     <sheet name="Side Table" sheetId="7" r:id="rId7"/>
     <sheet name="Debt Service" sheetId="8" r:id="rId8"/>
-    <sheet name="DSCR Notes" sheetId="9" r:id="rId9"/>
-    <sheet name="Lists" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet name="Reserves" sheetId="9" r:id="rId9"/>
+    <sheet name="DSCR Notes" sheetId="10" r:id="rId10"/>
+    <sheet name="Lists" sheetId="11" state="hidden" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="ChartNames">OFFSET(Lists!$A$2,0,0,MAX(1,COUNTIF(Lists!$A$2:$A$101,"?*")),1)</definedName>
@@ -347,41 +348,55 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown beside the cash flow table on page 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
+          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown on page 2 below the reserves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -393,6 +408,55 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="90" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heading</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Seasonality</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q1 and Q4 coverage falls below 1.0x on a stand-alone basis every year; the covenants test on an LTM basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Next test</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 2026 test at September 30, 2026.  Distributions require 1.20x LTM.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1449,7 +1513,7 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lock-up DSCR</t>
+          <t xml:space="preserve">Distribution lock-up DSCR</t>
         </is>
       </c>
       <c r="B27" s="8">
@@ -1457,7 +1521,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution lock-up covenant, e.g. 1.20.  Drawn as a reference line; leave blank for none.</t>
+          <t xml:space="preserve">Distribution lock-up covenant, e.g. 1.20.  Drawn as a reference line.  Leave blank and it does not appear anywhere.</t>
         </is>
       </c>
     </row>
@@ -1472,37 +1536,54 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Default covenant, e.g. 1.10.  Drawn as a reference line; leave blank for none.</t>
+          <t xml:space="preserve">Default covenant, e.g. 1.10.  Drawn as a reference line.  Leave blank and it does not appear anywhere.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cash flow units</t>
+          <t xml:space="preserve">Reserves title</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">$MM</t>
+          <t xml:space="preserve">DSR and O&amp;M Reserves</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units label for page 2, e.g. $MM or $000s.</t>
+          <t xml:space="preserve">Header of the reserves box on page 2 (below the DSCR chart).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Cash flow units</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$MM</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units label for page 2, e.g. $MM or $000s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Cash flow decimals</t>
         </is>
       </c>
-      <c r="B30" s="8">
+      <c r="B31" s="8">
         <v>2</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Decimals in the page 2 cash flow table.</t>
         </is>
@@ -2716,45 +2797,63 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="90" customWidth="1"/>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heading</t>
+          <t xml:space="preserve">Reserve</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text</t>
+          <t xml:space="preserve">Required</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Balance available</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seasonality</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Q1 and Q4 coverage falls below 1.0x on a stand-alone basis every year; the covenants test on an LTM basis.</t>
-        </is>
+          <t xml:space="preserve">Debt service reserve</t>
+        </is>
+      </c>
+      <c r="B2" s="10">
+        <v>8.55</v>
+      </c>
+      <c r="C2" s="10">
+        <v>8.62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Next test</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Q3 2026 test at September 30, 2026.  Distributions require 1.20x LTM.</t>
-        </is>
-      </c>
+          <t xml:space="preserve">O&amp;M reserve</t>
+        </is>
+      </c>
+      <c r="B3" s="10">
+        <v>2.1</v>
+      </c>
+      <c r="C3" s="10">
+        <v>1.85</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Dashboard builder: Table actuals as live Excel formulas
Month Actual and YTD Actual on the Table tab are now formulas (with
cached results) instead of a "(from Charts)" placeholder: SUMIFS /
SUMPRODUCT over the Charts tab keyed on From Chart, From Component,
YTD Method and the CurYear / CurMonthNum names that point at Settings.
O&M expense defaults to Revenue - Operating income.  The builder uses
the cell's value, so a typed override wins; it recomputes from the
Charts tab only when the cell is empty or an error.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -19,6 +19,8 @@
   </sheets>
   <definedNames>
     <definedName name="ChartNames">OFFSET(Lists!$A$2,0,0,MAX(1,COUNTIF(Lists!$A$2:$A$101,"?*")),1)</definedName>
+    <definedName name="CurYear">Settings!$B$6</definedName>
+    <definedName name="CurMonthNum">IF(ISNUMBER(Settings!$B$8),Settings!$B$8,MATCH(LEFT(Settings!$B$8,3),{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -131,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -154,6 +156,9 @@
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -285,118 +290,132 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Pick a chart in "From Chart" (dropdown) to fill Month Actual and YTD Actual from the Charts tab automatically</t>
+          <t xml:space="preserve">               Month Actual and YTD Actual (black cells) are formulas: rows with a "From Chart" sum that chart on the Charts tab for the</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">               (add a "From Component" to use just one component, e.g. Contracted).  Leave "From Chart" blank to type the actuals yourself.</t>
+          <t xml:space="preserve">               Current year, for the Current month and Jan through it (add a "From Component" to use one component, e.g. Contracted).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
+          <t xml:space="preserve">               O&amp;M expense defaults to Revenue - Operating income.  Type a number over any formula to override it; the PDF uses the cell value.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
+          <t xml:space="preserve">               Rows with no "From Chart" and no formula: type the actuals yourself.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
+          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
+          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Service  -  quarterly cash flow for page 2.  One column per quarter, oldest on the left.  Role: Revenue, Expense or Debt service.</t>
+          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  CFADS = Revenue - Expenses.  DSCR = CFADS / Debt service.</t>
+          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">               LTM DSCR = last 4 quarters of CFADS / last 4 quarters of debt service.  Add any expense or debt service rows you need.</t>
+          <t xml:space="preserve">Debt Service  -  quarterly cash flow for page 2.  One column per quarter, oldest on the left.  Role: Revenue, Expense or Debt service.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  CFADS = Revenue - Expenses.  DSCR = CFADS / Debt service.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+          <t xml:space="preserve">               LTM DSCR = last 4 quarters of CFADS / last 4 quarters of debt service.  Add any expense or debt service rows you need.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown on page 2 below the reserves.</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -2211,18 +2230,16 @@
       </c>
       <c r="I2" s="8"/>
       <c r="J2" s="8"/>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(from Charts)</t>
-        </is>
+      <c r="K2" s="13">
+        <f>IF($C2="",SUMIFS(INDEX(Charts!$E$2:$P$500,0,CurMonthNum),Charts!$A$2:$A$500,$B2,Charts!$C$2:$C$500,CurYear),SUMIFS(INDEX(Charts!$E$2:$P$500,0,CurMonthNum),Charts!$A$2:$A$500,$B2,Charts!$C$2:$C$500,CurYear,Charts!$B$2:$B$500,$C2))</f>
+        <v>47.2</v>
       </c>
       <c r="L2" s="9">
         <v>50.6</v>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(from Charts)</t>
-        </is>
+      <c r="M2" s="13">
+        <f>SUMPRODUCT((Charts!$A$2:$A$500=$B2)*(Charts!$C$2:$C$500=CurYear)*((($C2="")+(Charts!$B$2:$B$500=$C2))&gt;0)*(COLUMN(Charts!$E$1:$P$1)-COLUMN(Charts!$E$1)&lt;CurMonthNum),Charts!$E$2:$P$500)/IF($D2="Average",CurMonthNum,1)</f>
+        <v>326</v>
       </c>
       <c r="N2" s="9">
         <v>351.4</v>
@@ -2265,18 +2282,16 @@
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(from Charts)</t>
-        </is>
+      <c r="K3" s="14">
+        <f>IF($C3="",SUMIFS(INDEX(Charts!$E$2:$P$500,0,CurMonthNum),Charts!$A$2:$A$500,$B3,Charts!$C$2:$C$500,CurYear),SUMIFS(INDEX(Charts!$E$2:$P$500,0,CurMonthNum),Charts!$A$2:$A$500,$B3,Charts!$C$2:$C$500,CurYear,Charts!$B$2:$B$500,$C3))</f>
+        <v>3.92</v>
       </c>
       <c r="L3" s="10">
         <v>3.85</v>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(from Charts)</t>
-        </is>
+      <c r="M3" s="14">
+        <f>SUMPRODUCT((Charts!$A$2:$A$500=$B3)*(Charts!$C$2:$C$500=CurYear)*((($C3="")+(Charts!$B$2:$B$500=$C3))&gt;0)*(COLUMN(Charts!$E$1:$P$1)-COLUMN(Charts!$E$1)&lt;CurMonthNum),Charts!$E$2:$P$500)/IF($D3="Average",CurMonthNum,1)</f>
+        <v>23.97</v>
       </c>
       <c r="N3" s="10">
         <v>25.3</v>
@@ -2319,17 +2334,19 @@
         </is>
       </c>
       <c r="J4" s="8"/>
-      <c r="K4" s="10">
-        <v>0.86</v>
+      <c r="K4" s="14">
+        <f>K3-K5</f>
+        <v>1.85</v>
       </c>
       <c r="L4" s="10">
-        <v>0.74</v>
-      </c>
-      <c r="M4" s="10">
-        <v>6.12</v>
+        <v>1.54</v>
+      </c>
+      <c r="M4" s="14">
+        <f>M3-M5</f>
+        <v>14.38</v>
       </c>
       <c r="N4" s="10">
-        <v>6.4</v>
+        <v>13.68</v>
       </c>
     </row>
     <row r="5">
@@ -2373,18 +2390,16 @@
           <t xml:space="preserve">Y</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(from Charts)</t>
-        </is>
+      <c r="K5" s="14">
+        <f>IF($C5="",SUMIFS(INDEX(Charts!$E$2:$P$500,0,CurMonthNum),Charts!$A$2:$A$500,$B5,Charts!$C$2:$C$500,CurYear),SUMIFS(INDEX(Charts!$E$2:$P$500,0,CurMonthNum),Charts!$A$2:$A$500,$B5,Charts!$C$2:$C$500,CurYear,Charts!$B$2:$B$500,$C5))</f>
+        <v>2.07</v>
       </c>
       <c r="L5" s="10">
         <v>2.31</v>
       </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(from Charts)</t>
-        </is>
+      <c r="M5" s="14">
+        <f>SUMPRODUCT((Charts!$A$2:$A$500=$B5)*(Charts!$C$2:$C$500=CurYear)*((($C5="")+(Charts!$B$2:$B$500=$C5))&gt;0)*(COLUMN(Charts!$E$1:$P$1)-COLUMN(Charts!$E$1)&lt;CurMonthNum),Charts!$E$2:$P$500)/IF($D5="Average",CurMonthNum,1)</f>
+        <v>9.59</v>
       </c>
       <c r="N5" s="10">
         <v>11.62</v>

</xml_diff>

<commit_message>
Dashboard builder: EV Basis footnotes for pro-rated EV Case values
New Table column EV Basis (Monthly / Pro-rated quarterly / semi-annual /
annual).  Pro-rated rows get a letter marker on both EV Case cells and
one note per basis under the table, e.g. "EV Case pro-rated from
quarterly figures on a straight-line monthly basis; it does not reflect
seasonality within the quarter."  Settings > Pro-rated note overrides the
wording ({basis}, {period}, {comparison} placeholders).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -318,104 +318,118 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
+          <t xml:space="preserve">               "EV Basis": if the EV Case values were pro-rated from quarterly, semi-annual or annual figures, pick that here.  The EV Case</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
+          <t xml:space="preserve">               values get a small letter (a, b, ...) and a footnote under the table explains it.  Monthly (the default) adds nothing.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
+          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
+          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Service  -  quarterly cash flow for page 2.  One column per quarter, oldest on the left.  Role: Revenue, Expense or Debt service.</t>
+          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  CFADS = Revenue - Expenses.  DSCR = CFADS / Debt service.</t>
+          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">               LTM DSCR = last 4 quarters of CFADS / last 4 quarters of debt service.  Add any expense or debt service rows you need.</t>
+          <t xml:space="preserve">Debt Service  -  quarterly cash flow for page 2.  One column per quarter, oldest on the left.  Role: Revenue, Expense or Debt service.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  CFADS = Revenue - Expenses.  DSCR = CFADS / Debt service.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+          <t xml:space="preserve">               LTM DSCR = last 4 quarters of CFADS / last 4 quarters of debt service.  Add any expense or debt service rows you need.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown on page 2 below the reserves.</t>
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -1483,126 +1497,139 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Include DSCR page</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Auto</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Pro-rated note</t>
+        </is>
+      </c>
+      <c r="B24" s="8"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auto = add page 2 (Debt Service Coverage) when the Debt Service tab has data.  Yes / No to force it.</t>
+          <t xml:space="preserve">Optional wording for the EV Basis footnote under the table.  Blank = "EV Case pro-rated from quarterly figures on a straight-line monthly basis; it does not reflect seasonality within the quarter."  You can use {basis} (quarterly / semi-annual / annual), {period} (quarter / half-year / year) and {comparison} (the Comparison label).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSCR page title</t>
+          <t xml:space="preserve">Include DSCR page</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Service Coverage - LTM Basis</t>
+          <t xml:space="preserve">Auto</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header above the DSCR charts on page 2.</t>
+          <t xml:space="preserve">Auto = add page 2 (Debt Service Coverage) when the Debt Service tab has data.  Yes / No to force it.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quarters shown</t>
-        </is>
-      </c>
-      <c r="B26" s="8">
-        <v>4</v>
+          <t xml:space="preserve">DSCR page title</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt Service Coverage - LTM Basis</t>
+        </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">How many of the most recent quarters page 2 shows (1-8).  Enter 3 extra older quarters to show an LTM DSCR for every quarter shown.</t>
+          <t xml:space="preserve">Header above the DSCR charts on page 2.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution lock-up DSCR</t>
+          <t xml:space="preserve">Quarters shown</t>
         </is>
       </c>
       <c r="B27" s="8">
-        <v>1.2</v>
+        <v>4</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Distribution lock-up covenant, e.g. 1.20.  Drawn as a reference line.  Leave blank and it does not appear anywhere.</t>
+          <t xml:space="preserve">How many of the most recent quarters page 2 shows (1-8).  Enter 3 extra older quarters to show an LTM DSCR for every quarter shown.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Default DSCR</t>
+          <t xml:space="preserve">Distribution lock-up DSCR</t>
         </is>
       </c>
       <c r="B28" s="8">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Default covenant, e.g. 1.10.  Drawn as a reference line.  Leave blank and it does not appear anywhere.</t>
+          <t xml:space="preserve">Distribution lock-up covenant, e.g. 1.20.  Drawn as a reference line.  Leave blank and it does not appear anywhere.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserves title</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DSR and O&amp;M Reserves</t>
-        </is>
+          <t xml:space="preserve">Default DSCR</t>
+        </is>
+      </c>
+      <c r="B29" s="8">
+        <v>1.1</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header of the reserves box on page 2 (below the DSCR chart).</t>
+          <t xml:space="preserve">Default covenant, e.g. 1.10.  Drawn as a reference line.  Leave blank and it does not appear anywhere.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cash flow units</t>
+          <t xml:space="preserve">Reserves title</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">$MM</t>
+          <t xml:space="preserve">DSR and O&amp;M Reserves</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units label for page 2, e.g. $MM or $000s.</t>
+          <t xml:space="preserve">Header of the reserves box on page 2 (below the DSCR chart).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Cash flow units</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$MM</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units label for page 2, e.g. $MM or $000s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">Cash flow decimals</t>
         </is>
       </c>
-      <c r="B31" s="8">
+      <c r="B32" s="8">
         <v>2</v>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Decimals in the page 2 cash flow table.</t>
         </is>
@@ -1628,7 +1655,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B23">
       <formula1>"Letter,A4"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B25">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2123,6 +2150,7 @@
     <col min="12" max="12" width="15" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2194,6 +2222,11 @@
       <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">YTD EV Case</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EV Basis</t>
         </is>
       </c>
     </row>
@@ -2244,6 +2277,11 @@
       <c r="N2" s="9">
         <v>351.4</v>
       </c>
+      <c r="O2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monthly</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -2296,6 +2334,11 @@
       <c r="N3" s="10">
         <v>25.3</v>
       </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monthly</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -2348,6 +2391,11 @@
       <c r="N4" s="10">
         <v>13.68</v>
       </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pro-rated annual</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -2404,9 +2452,14 @@
       <c r="N5" s="10">
         <v>11.62</v>
       </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monthly</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B200">
       <formula1>ChartNames</formula1>
     </dataValidation>
@@ -2421,6 +2474,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J200">
       <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O200">
+      <formula1>"Monthly,Pro-rated quarterly,Pro-rated semi-annual,Pro-rated annual"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Dashboard builder: Debt Service tab calculates down to CFADS
The example workbooks' Debt Service tab now has Calculated formula rows:
Total O&M costs (all Expense rows), CFADS (Revenue - Total O&M costs),
Total debt service costs (all Debt service rows), DSCR - quarter and
DSCR - LTM.  Totals use SUMIF on the Role column, so a row inserted
anywhere with the right Role is included.  The builder skips Calculated
rows and recomputes from the inputs; page 2's cash flow table gains a
Total O&M costs line and says Total debt service costs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -28,9 +28,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -133,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -159,6 +160,8 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -367,69 +370,83 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  CFADS = Revenue - Expenses.  DSCR = CFADS / Debt service.</t>
+          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  The black "Calculated" rows do the math: Total O&amp;M costs = all Expense</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">               LTM DSCR = last 4 quarters of CFADS / last 4 quarters of debt service.  Add any expense or debt service rows you need.</t>
+          <t xml:space="preserve">               rows; CFADS = Revenue - Total O&amp;M costs; Total debt service costs = all Debt service rows; DSCR = CFADS / debt service;</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+          <t xml:space="preserve">               DSCR - LTM = last 4 quarters of CFADS / last 4 quarters of debt service.  To add a line (e.g. LC fees), insert a row</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+          <t xml:space="preserve">               anywhere and set its Role; the totals pick it up.  The PDF recalculates from the input rows, so it always matches.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown on page 2 below the reserves.</t>
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -2767,97 +2784,277 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total O&amp;M costs</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",C$2:C$200)</f>
+        <v>2.43</v>
+      </c>
+      <c r="D6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",D$2:D$200)</f>
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",E$2:E$200)</f>
+        <v>2.66</v>
+      </c>
+      <c r="F6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",F$2:F$200)</f>
+        <v>2.78</v>
+      </c>
+      <c r="G6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",G$2:G$200)</f>
+        <v>2.55</v>
+      </c>
+      <c r="H6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",H$2:H$200)</f>
+        <v>2.64</v>
+      </c>
+      <c r="I6" s="15">
+        <f>SUMIF($B$2:$B$200,"Expense",I$2:I$200)</f>
+        <v>2.83</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CFADS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",C$2:C$200)-SUMIF($B$2:$B$200,"Expense",C$2:C$200)</f>
+        <v>2.88</v>
+      </c>
+      <c r="D7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",D$2:D$200)-SUMIF($B$2:$B$200,"Expense",D$2:D$200)</f>
+        <v>3.12</v>
+      </c>
+      <c r="E7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",E$2:E$200)-SUMIF($B$2:$B$200,"Expense",E$2:E$200)</f>
+        <v>7.38</v>
+      </c>
+      <c r="F7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",F$2:F$200)-SUMIF($B$2:$B$200,"Expense",F$2:F$200)</f>
+        <v>7.74</v>
+      </c>
+      <c r="G7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",G$2:G$200)-SUMIF($B$2:$B$200,"Expense",G$2:G$200)</f>
+        <v>3.38</v>
+      </c>
+      <c r="H7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",H$2:H$200)-SUMIF($B$2:$B$200,"Expense",H$2:H$200)</f>
+        <v>3.44</v>
+      </c>
+      <c r="I7" s="15">
+        <f>SUMIF($B$2:$B$200,"Revenue",I$2:I$200)-SUMIF($B$2:$B$200,"Expense",I$2:I$200)</f>
+        <v>7.78</v>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Principal</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C6" s="10">
+      <c r="C9" s="10">
         <v>2.4</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D9" s="10">
         <v>2.42</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E9" s="10">
         <v>2.48</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F9" s="10">
         <v>2.51</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G9" s="10">
         <v>2.57</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H9" s="10">
         <v>2.62</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I9" s="10">
         <v>2.68</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C7" s="10">
+      <c r="C10" s="10">
         <v>1.91</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D10" s="10">
         <v>1.86</v>
       </c>
-      <c r="E7" s="10">
+      <c r="E10" s="10">
         <v>1.81</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F10" s="10">
         <v>1.76</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G10" s="10">
         <v>1.7</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H10" s="10">
         <v>1.65</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I10" s="10">
         <v>1.6</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total debt service costs</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",C$2:C$200)</f>
+        <v>4.31</v>
+      </c>
+      <c r="D11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",D$2:D$200)</f>
+        <v>4.28</v>
+      </c>
+      <c r="E11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",E$2:E$200)</f>
+        <v>4.29</v>
+      </c>
+      <c r="F11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",F$2:F$200)</f>
+        <v>4.27</v>
+      </c>
+      <c r="G11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",G$2:G$200)</f>
+        <v>4.27</v>
+      </c>
+      <c r="H11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",H$2:H$200)</f>
+        <v>4.27</v>
+      </c>
+      <c r="I11" s="15">
+        <f>SUMIF($B$2:$B$200,"Debt service",I$2:I$200)</f>
+        <v>4.28</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DSCR - quarter</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C13" s="16">
+        <f>IFERROR(C7/C11,"")</f>
+        <v>0.668213</v>
+      </c>
+      <c r="D13" s="16">
+        <f>IFERROR(D7/D11,"")</f>
+        <v>0.728972</v>
+      </c>
+      <c r="E13" s="16">
+        <f>IFERROR(E7/E11,"")</f>
+        <v>1.72028</v>
+      </c>
+      <c r="F13" s="16">
+        <f>IFERROR(F7/F11,"")</f>
+        <v>1.812646</v>
+      </c>
+      <c r="G13" s="16">
+        <f>IFERROR(G7/G11,"")</f>
+        <v>0.791569</v>
+      </c>
+      <c r="H13" s="16">
+        <f>IFERROR(H7/H11,"")</f>
+        <v>0.805621</v>
+      </c>
+      <c r="I13" s="16">
+        <f>IFERROR(I7/I11,"")</f>
+        <v>1.817757</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DSCR - LTM</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="D14" s="16" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E14" s="16" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="F14" s="16">
+        <f>IFERROR(SUM(C7:F7)/SUM(C11:F11),"")</f>
+        <v>1.231487</v>
+      </c>
+      <c r="G14" s="16">
+        <f>IFERROR(SUM(D7:G7)/SUM(D11:G11),"")</f>
+        <v>1.263589</v>
+      </c>
+      <c r="H14" s="16">
+        <f>IFERROR(SUM(E7:H7)/SUM(E11:H11),"")</f>
+        <v>1.283041</v>
+      </c>
+      <c r="I14" s="16">
+        <f>IFERROR(SUM(F7:I7)/SUM(F11:I11),"")</f>
+        <v>1.307197</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B100">
-      <formula1>"Revenue,Expense,Debt service"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B200">
+      <formula1>"Revenue,Expense,Debt service,Calculated"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Dashboard builder: blank row between revenue and expenses on the Debt Service tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -2684,43 +2684,11 @@
         <v>10.61</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">O&amp;M</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Expense</t>
-        </is>
-      </c>
-      <c r="C3" s="10">
-        <v>1.92</v>
-      </c>
-      <c r="D3" s="10">
-        <v>2.01</v>
-      </c>
-      <c r="E3" s="10">
-        <v>2.08</v>
-      </c>
-      <c r="F3" s="10">
-        <v>2.17</v>
-      </c>
-      <c r="G3" s="10">
-        <v>2.03</v>
-      </c>
-      <c r="H3" s="10">
-        <v>2.11</v>
-      </c>
-      <c r="I3" s="10">
-        <v>2.19</v>
-      </c>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Property taxes</t>
+          <t xml:space="preserve">O&amp;M</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -2729,325 +2697,358 @@
         </is>
       </c>
       <c r="C4" s="10">
-        <v>0.4</v>
+        <v>1.92</v>
       </c>
       <c r="D4" s="10">
-        <v>0.4</v>
+        <v>2.01</v>
       </c>
       <c r="E4" s="10">
-        <v>0.4</v>
+        <v>2.08</v>
       </c>
       <c r="F4" s="10">
-        <v>0.4</v>
+        <v>2.17</v>
       </c>
       <c r="G4" s="10">
-        <v>0.42</v>
+        <v>2.03</v>
       </c>
       <c r="H4" s="10">
-        <v>0.45</v>
+        <v>2.11</v>
       </c>
       <c r="I4" s="10">
-        <v>0.45</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Property taxes</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Expense</t>
+        </is>
+      </c>
+      <c r="C5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="D5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="E5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="F5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="G5" s="10">
+        <v>0.42</v>
+      </c>
+      <c r="H5" s="10">
+        <v>0.45</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Other taxes</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C5" s="10">
+      <c r="C6" s="10">
         <v>0.11</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D6" s="10">
         <v>0.09</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E6" s="10">
         <v>0.18</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F6" s="10">
         <v>0.21</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G6" s="10">
         <v>0.1</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H6" s="10">
         <v>0.08</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I6" s="10">
         <v>0.19</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Total O&amp;M costs</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C6" s="15">
+      <c r="C7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",C$2:C$200)</f>
         <v>2.43</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",D$2:D$200)</f>
         <v>2.5</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",E$2:E$200)</f>
         <v>2.66</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",F$2:F$200)</f>
         <v>2.78</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",G$2:G$200)</f>
         <v>2.55</v>
       </c>
-      <c r="H6" s="15">
+      <c r="H7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",H$2:H$200)</f>
         <v>2.64</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I7" s="15">
         <f>SUMIF($B$2:$B$200,"Expense",I$2:I$200)</f>
         <v>2.83</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">CFADS</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C7" s="15">
+      <c r="C8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",C$2:C$200)-SUMIF($B$2:$B$200,"Expense",C$2:C$200)</f>
         <v>2.88</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",D$2:D$200)-SUMIF($B$2:$B$200,"Expense",D$2:D$200)</f>
         <v>3.12</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",E$2:E$200)-SUMIF($B$2:$B$200,"Expense",E$2:E$200)</f>
         <v>7.38</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",F$2:F$200)-SUMIF($B$2:$B$200,"Expense",F$2:F$200)</f>
         <v>7.74</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",G$2:G$200)-SUMIF($B$2:$B$200,"Expense",G$2:G$200)</f>
         <v>3.38</v>
       </c>
-      <c r="H7" s="15">
+      <c r="H8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",H$2:H$200)-SUMIF($B$2:$B$200,"Expense",H$2:H$200)</f>
         <v>3.44</v>
       </c>
-      <c r="I7" s="15">
+      <c r="I8" s="15">
         <f>SUMIF($B$2:$B$200,"Revenue",I$2:I$200)-SUMIF($B$2:$B$200,"Expense",I$2:I$200)</f>
         <v>7.78</v>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Principal</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Debt service</t>
-        </is>
-      </c>
-      <c r="C9" s="10">
-        <v>2.4</v>
-      </c>
-      <c r="D9" s="10">
-        <v>2.42</v>
-      </c>
-      <c r="E9" s="10">
-        <v>2.48</v>
-      </c>
-      <c r="F9" s="10">
-        <v>2.51</v>
-      </c>
-      <c r="G9" s="10">
-        <v>2.57</v>
-      </c>
-      <c r="H9" s="10">
-        <v>2.62</v>
-      </c>
-      <c r="I9" s="10">
-        <v>2.68</v>
-      </c>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Principal</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service</t>
+        </is>
+      </c>
+      <c r="C10" s="10">
+        <v>2.4</v>
+      </c>
+      <c r="D10" s="10">
+        <v>2.42</v>
+      </c>
+      <c r="E10" s="10">
+        <v>2.48</v>
+      </c>
+      <c r="F10" s="10">
+        <v>2.51</v>
+      </c>
+      <c r="G10" s="10">
+        <v>2.57</v>
+      </c>
+      <c r="H10" s="10">
+        <v>2.62</v>
+      </c>
+      <c r="I10" s="10">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Interest</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C10" s="10">
+      <c r="C11" s="10">
         <v>1.91</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D11" s="10">
         <v>1.86</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E11" s="10">
         <v>1.81</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F11" s="10">
         <v>1.76</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G11" s="10">
         <v>1.7</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H11" s="10">
         <v>1.65</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I11" s="10">
         <v>1.6</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Total debt service costs</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C11" s="15">
+      <c r="C12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",C$2:C$200)</f>
         <v>4.31</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",D$2:D$200)</f>
         <v>4.28</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",E$2:E$200)</f>
         <v>4.29</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",F$2:F$200)</f>
         <v>4.27</v>
       </c>
-      <c r="G11" s="15">
+      <c r="G12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",G$2:G$200)</f>
         <v>4.27</v>
       </c>
-      <c r="H11" s="15">
+      <c r="H12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",H$2:H$200)</f>
         <v>4.27</v>
       </c>
-      <c r="I11" s="15">
+      <c r="I12" s="15">
         <f>SUMIF($B$2:$B$200,"Debt service",I$2:I$200)</f>
         <v>4.28</v>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DSCR - quarter</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Calculated</t>
-        </is>
-      </c>
-      <c r="C13" s="16">
-        <f>IFERROR(C7/C11,"")</f>
-        <v>0.668213</v>
-      </c>
-      <c r="D13" s="16">
-        <f>IFERROR(D7/D11,"")</f>
-        <v>0.728972</v>
-      </c>
-      <c r="E13" s="16">
-        <f>IFERROR(E7/E11,"")</f>
-        <v>1.72028</v>
-      </c>
-      <c r="F13" s="16">
-        <f>IFERROR(F7/F11,"")</f>
-        <v>1.812646</v>
-      </c>
-      <c r="G13" s="16">
-        <f>IFERROR(G7/G11,"")</f>
-        <v>0.791569</v>
-      </c>
-      <c r="H13" s="16">
-        <f>IFERROR(H7/H11,"")</f>
-        <v>0.805621</v>
-      </c>
-      <c r="I13" s="16">
-        <f>IFERROR(I7/I11,"")</f>
-        <v>1.817757</v>
-      </c>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">DSCR - quarter</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C14" s="16">
+        <f>IFERROR(C8/C12,"")</f>
+        <v>0.668213</v>
+      </c>
+      <c r="D14" s="16">
+        <f>IFERROR(D8/D12,"")</f>
+        <v>0.728972</v>
+      </c>
+      <c r="E14" s="16">
+        <f>IFERROR(E8/E12,"")</f>
+        <v>1.72028</v>
+      </c>
+      <c r="F14" s="16">
+        <f>IFERROR(F8/F12,"")</f>
+        <v>1.812646</v>
+      </c>
+      <c r="G14" s="16">
+        <f>IFERROR(G8/G12,"")</f>
+        <v>0.791569</v>
+      </c>
+      <c r="H14" s="16">
+        <f>IFERROR(H8/H12,"")</f>
+        <v>0.805621</v>
+      </c>
+      <c r="I14" s="16">
+        <f>IFERROR(I8/I12,"")</f>
+        <v>1.817757</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR - LTM</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C14" s="16" t="str">
+      <c r="C15" s="16" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="D14" s="16" t="str">
+      <c r="D15" s="16" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="E14" s="16" t="str">
+      <c r="E15" s="16" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F14" s="16">
-        <f>IFERROR(SUM(C7:F7)/SUM(C11:F11),"")</f>
+      <c r="F15" s="16">
+        <f>IFERROR(SUM(C8:F8)/SUM(C12:F12),"")</f>
         <v>1.231487</v>
       </c>
-      <c r="G14" s="16">
-        <f>IFERROR(SUM(D7:G7)/SUM(D11:G11),"")</f>
+      <c r="G15" s="16">
+        <f>IFERROR(SUM(D8:G8)/SUM(D12:G12),"")</f>
         <v>1.263589</v>
       </c>
-      <c r="H14" s="16">
-        <f>IFERROR(SUM(E7:H7)/SUM(E11:H11),"")</f>
+      <c r="H15" s="16">
+        <f>IFERROR(SUM(E8:H8)/SUM(E12:H12),"")</f>
         <v>1.283041</v>
       </c>
-      <c r="I14" s="16">
-        <f>IFERROR(SUM(F7:I7)/SUM(F11:I11),"")</f>
+      <c r="I15" s="16">
+        <f>IFERROR(SUM(F8:I8)/SUM(F12:I12),"")</f>
         <v>1.307197</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard builder: Debt Service as a running history; page 2 follows Current month
- The Debt Service tab holds a fixed quarterly history (Q1 2024 to Q4
  2027) filled in as quarters close.  The builder places each column on
  a timeline and shows the last completed quarter before the Current
  month's quarter plus the 3 before it (Aug -> through Q2, Dec -> through
  Q3), skipping LTM across gaps; later quarters are noted, not shown.
- Fix: the Calculated rows used whole-column SUMIF ranges that included
  their own cells, a circular reference in Excel.  Each total now sums
  only its own block of input rows.
- New blue info messages for expected, non-problem notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -363,90 +363,104 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Service  -  quarterly cash flow for page 2.  One column per quarter, oldest on the left.  Role: Revenue, Expense or Debt service.</t>
+          <t xml:space="preserve">Debt Service  -  a running quarterly history for page 2: one column per quarter (Q1 2024 to Q4 2027).  Fill in each quarter when it closes;</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Enter expenses and debt service as positive numbers.  The black "Calculated" rows do the math: Total O&amp;M costs = all Expense</t>
+          <t xml:space="preserve">               nothing ever needs shifting.  Page 2 shows the last completed quarter before the Current month's quarter and the 3 before it</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">               rows; CFADS = Revenue - Total O&amp;M costs; Total debt service costs = all Debt service rows; DSCR = CFADS / debt service;</t>
+          <t xml:space="preserve">               (Current month Aug -&gt; through Q2; Dec -&gt; through Q3).  Add more quarters by adding columns with labels like "Q1 2028".</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">               DSCR - LTM = last 4 quarters of CFADS / last 4 quarters of debt service.  To add a line (e.g. LC fees), insert a row</t>
+          <t xml:space="preserve">               Role: Revenue, Expense or Debt service.  Enter expenses and debt service as positive numbers.  The black "Calculated</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">               anywhere and set its Role; the totals pick it up.  The PDF recalculates from the input rows, so it always matches.</t>
+          <t xml:space="preserve">               rows do the math: Total O&amp;M costs, CFADS = Revenue - Total O&amp;M costs, Total debt service costs, DSCR, and DSCR - LTM</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+          <t xml:space="preserve">               (last 4 quarters of CFADS / last 4 quarters of debt service).  To add a line (e.g. LC fees), insert the row between two</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+          <t xml:space="preserve">               rows of the same block so the totals' ranges grow to include it.  The PDF recalculates from the input rows.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown on page 2 below the reserves.</t>
         </is>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+    <row r="39"/>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -2595,13 +2609,22 @@
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="15" max="15" width="10" customWidth="1"/>
+    <col min="16" max="16" width="10" customWidth="1"/>
+    <col min="17" max="17" width="10" customWidth="1"/>
+    <col min="18" max="18" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2617,37 +2640,82 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Q1 2024</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q2 2024</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 2024</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Q4 2024</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Q1 2025</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Q2 2025</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Q3 2025</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Q4 2025</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Q1 2026</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Q2 2026</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 2026</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4 2026</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q1 2027</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q2 2027</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q3 2027</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q4 2027</t>
         </is>
       </c>
     </row>
@@ -2662,27 +2730,38 @@
           <t xml:space="preserve">Revenue</t>
         </is>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10">
         <v>5.31</v>
       </c>
-      <c r="D2" s="10">
+      <c r="G2" s="10">
         <v>5.62</v>
       </c>
-      <c r="E2" s="10">
+      <c r="H2" s="10">
         <v>10.04</v>
       </c>
-      <c r="F2" s="10">
+      <c r="I2" s="10">
         <v>10.52</v>
       </c>
-      <c r="G2" s="10">
+      <c r="J2" s="10">
         <v>5.93</v>
       </c>
-      <c r="H2" s="10">
+      <c r="K2" s="10">
         <v>6.08</v>
       </c>
-      <c r="I2" s="10">
+      <c r="L2" s="10">
         <v>10.61</v>
       </c>
+      <c r="M2" s="10">
+        <v>10.94</v>
+      </c>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="10"/>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
     </row>
     <row r="3"/>
     <row r="4">
@@ -2696,27 +2775,38 @@
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10">
         <v>1.92</v>
       </c>
-      <c r="D4" s="10">
+      <c r="G4" s="10">
         <v>2.01</v>
       </c>
-      <c r="E4" s="10">
+      <c r="H4" s="10">
         <v>2.08</v>
       </c>
-      <c r="F4" s="10">
+      <c r="I4" s="10">
         <v>2.17</v>
       </c>
-      <c r="G4" s="10">
+      <c r="J4" s="10">
         <v>2.03</v>
       </c>
-      <c r="H4" s="10">
+      <c r="K4" s="10">
         <v>2.11</v>
       </c>
-      <c r="I4" s="10">
+      <c r="L4" s="10">
         <v>2.19</v>
       </c>
+      <c r="M4" s="10">
+        <v>2.24</v>
+      </c>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -2729,27 +2819,38 @@
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C5" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="D5" s="10">
-        <v>0.4</v>
-      </c>
-      <c r="E5" s="10">
-        <v>0.4</v>
-      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="10">
         <v>0.4</v>
       </c>
       <c r="G5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="H5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0.4</v>
+      </c>
+      <c r="J5" s="10">
         <v>0.42</v>
       </c>
-      <c r="H5" s="10">
+      <c r="K5" s="10">
         <v>0.45</v>
       </c>
-      <c r="I5" s="10">
+      <c r="L5" s="10">
         <v>0.45</v>
       </c>
+      <c r="M5" s="10">
+        <v>0.45</v>
+      </c>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -2762,27 +2863,38 @@
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10">
         <v>0.11</v>
       </c>
-      <c r="D6" s="10">
+      <c r="G6" s="10">
         <v>0.09</v>
       </c>
-      <c r="E6" s="10">
+      <c r="H6" s="10">
         <v>0.18</v>
       </c>
-      <c r="F6" s="10">
+      <c r="I6" s="10">
         <v>0.21</v>
       </c>
-      <c r="G6" s="10">
+      <c r="J6" s="10">
         <v>0.1</v>
       </c>
-      <c r="H6" s="10">
+      <c r="K6" s="10">
         <v>0.08</v>
       </c>
-      <c r="I6" s="10">
+      <c r="L6" s="10">
         <v>0.19</v>
       </c>
+      <c r="M6" s="10">
+        <v>0.22</v>
+      </c>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -2795,33 +2907,69 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",C$2:C$200)</f>
+      <c r="C7" s="15" t="str">
+        <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C4:C6))</f>
+        <v/>
+      </c>
+      <c r="D7" s="15" t="str">
+        <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D4:D6))</f>
+        <v/>
+      </c>
+      <c r="E7" s="15" t="str">
+        <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E4:E6))</f>
+        <v/>
+      </c>
+      <c r="F7" s="15">
+        <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F4:F6))</f>
         <v>2.43</v>
       </c>
-      <c r="D7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",D$2:D$200)</f>
+      <c r="G7" s="15">
+        <f>IF(COUNT(G2:G3,G4:G6,G10:G11)=0,"",SUM(G4:G6))</f>
         <v>2.5</v>
       </c>
-      <c r="E7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",E$2:E$200)</f>
+      <c r="H7" s="15">
+        <f>IF(COUNT(H2:H3,H4:H6,H10:H11)=0,"",SUM(H4:H6))</f>
         <v>2.66</v>
       </c>
-      <c r="F7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",F$2:F$200)</f>
+      <c r="I7" s="15">
+        <f>IF(COUNT(I2:I3,I4:I6,I10:I11)=0,"",SUM(I4:I6))</f>
         <v>2.78</v>
       </c>
-      <c r="G7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",G$2:G$200)</f>
+      <c r="J7" s="15">
+        <f>IF(COUNT(J2:J3,J4:J6,J10:J11)=0,"",SUM(J4:J6))</f>
         <v>2.55</v>
       </c>
-      <c r="H7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",H$2:H$200)</f>
+      <c r="K7" s="15">
+        <f>IF(COUNT(K2:K3,K4:K6,K10:K11)=0,"",SUM(K4:K6))</f>
         <v>2.64</v>
       </c>
-      <c r="I7" s="15">
-        <f>SUMIF($B$2:$B$200,"Expense",I$2:I$200)</f>
+      <c r="L7" s="15">
+        <f>IF(COUNT(L2:L3,L4:L6,L10:L11)=0,"",SUM(L4:L6))</f>
         <v>2.83</v>
+      </c>
+      <c r="M7" s="15">
+        <f>IF(COUNT(M2:M3,M4:M6,M10:M11)=0,"",SUM(M4:M6))</f>
+        <v>2.91</v>
+      </c>
+      <c r="N7" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N6,N10:N11)=0,"",SUM(N4:N6))</f>
+        <v/>
+      </c>
+      <c r="O7" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O6,O10:O11)=0,"",SUM(O4:O6))</f>
+        <v/>
+      </c>
+      <c r="P7" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P6,P10:P11)=0,"",SUM(P4:P6))</f>
+        <v/>
+      </c>
+      <c r="Q7" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q6,Q10:Q11)=0,"",SUM(Q4:Q6))</f>
+        <v/>
+      </c>
+      <c r="R7" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R6,R10:R11)=0,"",SUM(R4:R6))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -2835,33 +2983,69 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",C$2:C$200)-SUMIF($B$2:$B$200,"Expense",C$2:C$200)</f>
+      <c r="C8" s="15" t="str">
+        <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C2:C3)-C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="15" t="str">
+        <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D2:D3)-D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="15" t="str">
+        <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E2:E3)-E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="15">
+        <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F2:F3)-F7)</f>
         <v>2.88</v>
       </c>
-      <c r="D8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",D$2:D$200)-SUMIF($B$2:$B$200,"Expense",D$2:D$200)</f>
+      <c r="G8" s="15">
+        <f>IF(COUNT(G2:G3,G4:G6,G10:G11)=0,"",SUM(G2:G3)-G7)</f>
         <v>3.12</v>
       </c>
-      <c r="E8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",E$2:E$200)-SUMIF($B$2:$B$200,"Expense",E$2:E$200)</f>
+      <c r="H8" s="15">
+        <f>IF(COUNT(H2:H3,H4:H6,H10:H11)=0,"",SUM(H2:H3)-H7)</f>
         <v>7.38</v>
       </c>
-      <c r="F8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",F$2:F$200)-SUMIF($B$2:$B$200,"Expense",F$2:F$200)</f>
+      <c r="I8" s="15">
+        <f>IF(COUNT(I2:I3,I4:I6,I10:I11)=0,"",SUM(I2:I3)-I7)</f>
         <v>7.74</v>
       </c>
-      <c r="G8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",G$2:G$200)-SUMIF($B$2:$B$200,"Expense",G$2:G$200)</f>
+      <c r="J8" s="15">
+        <f>IF(COUNT(J2:J3,J4:J6,J10:J11)=0,"",SUM(J2:J3)-J7)</f>
         <v>3.38</v>
       </c>
-      <c r="H8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",H$2:H$200)-SUMIF($B$2:$B$200,"Expense",H$2:H$200)</f>
+      <c r="K8" s="15">
+        <f>IF(COUNT(K2:K3,K4:K6,K10:K11)=0,"",SUM(K2:K3)-K7)</f>
         <v>3.44</v>
       </c>
-      <c r="I8" s="15">
-        <f>SUMIF($B$2:$B$200,"Revenue",I$2:I$200)-SUMIF($B$2:$B$200,"Expense",I$2:I$200)</f>
+      <c r="L8" s="15">
+        <f>IF(COUNT(L2:L3,L4:L6,L10:L11)=0,"",SUM(L2:L3)-L7)</f>
         <v>7.78</v>
+      </c>
+      <c r="M8" s="15">
+        <f>IF(COUNT(M2:M3,M4:M6,M10:M11)=0,"",SUM(M2:M3)-M7)</f>
+        <v>8.03</v>
+      </c>
+      <c r="N8" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N6,N10:N11)=0,"",SUM(N2:N3)-N7)</f>
+        <v/>
+      </c>
+      <c r="O8" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O6,O10:O11)=0,"",SUM(O2:O3)-O7)</f>
+        <v/>
+      </c>
+      <c r="P8" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P6,P10:P11)=0,"",SUM(P2:P3)-P7)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q6,Q10:Q11)=0,"",SUM(Q2:Q3)-Q7)</f>
+        <v/>
+      </c>
+      <c r="R8" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R6,R10:R11)=0,"",SUM(R2:R3)-R7)</f>
+        <v/>
       </c>
     </row>
     <row r="9"/>
@@ -2876,27 +3060,38 @@
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10">
         <v>2.4</v>
       </c>
-      <c r="D10" s="10">
+      <c r="G10" s="10">
         <v>2.42</v>
       </c>
-      <c r="E10" s="10">
+      <c r="H10" s="10">
         <v>2.48</v>
       </c>
-      <c r="F10" s="10">
+      <c r="I10" s="10">
         <v>2.51</v>
       </c>
-      <c r="G10" s="10">
+      <c r="J10" s="10">
         <v>2.57</v>
       </c>
-      <c r="H10" s="10">
+      <c r="K10" s="10">
         <v>2.62</v>
       </c>
-      <c r="I10" s="10">
+      <c r="L10" s="10">
         <v>2.68</v>
       </c>
+      <c r="M10" s="10">
+        <v>2.74</v>
+      </c>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -2909,27 +3104,38 @@
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10">
         <v>1.91</v>
       </c>
-      <c r="D11" s="10">
+      <c r="G11" s="10">
         <v>1.86</v>
       </c>
-      <c r="E11" s="10">
+      <c r="H11" s="10">
         <v>1.81</v>
       </c>
-      <c r="F11" s="10">
+      <c r="I11" s="10">
         <v>1.76</v>
       </c>
-      <c r="G11" s="10">
+      <c r="J11" s="10">
         <v>1.7</v>
       </c>
-      <c r="H11" s="10">
+      <c r="K11" s="10">
         <v>1.65</v>
       </c>
-      <c r="I11" s="10">
+      <c r="L11" s="10">
         <v>1.6</v>
       </c>
+      <c r="M11" s="10">
+        <v>1.55</v>
+      </c>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -2942,33 +3148,69 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",C$2:C$200)</f>
+      <c r="C12" s="15" t="str">
+        <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C10:C11))</f>
+        <v/>
+      </c>
+      <c r="D12" s="15" t="str">
+        <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D10:D11))</f>
+        <v/>
+      </c>
+      <c r="E12" s="15" t="str">
+        <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E10:E11))</f>
+        <v/>
+      </c>
+      <c r="F12" s="15">
+        <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F10:F11))</f>
         <v>4.31</v>
       </c>
-      <c r="D12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",D$2:D$200)</f>
+      <c r="G12" s="15">
+        <f>IF(COUNT(G2:G3,G4:G6,G10:G11)=0,"",SUM(G10:G11))</f>
         <v>4.28</v>
       </c>
-      <c r="E12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",E$2:E$200)</f>
+      <c r="H12" s="15">
+        <f>IF(COUNT(H2:H3,H4:H6,H10:H11)=0,"",SUM(H10:H11))</f>
         <v>4.29</v>
       </c>
-      <c r="F12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",F$2:F$200)</f>
+      <c r="I12" s="15">
+        <f>IF(COUNT(I2:I3,I4:I6,I10:I11)=0,"",SUM(I10:I11))</f>
         <v>4.27</v>
       </c>
-      <c r="G12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",G$2:G$200)</f>
+      <c r="J12" s="15">
+        <f>IF(COUNT(J2:J3,J4:J6,J10:J11)=0,"",SUM(J10:J11))</f>
         <v>4.27</v>
       </c>
-      <c r="H12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",H$2:H$200)</f>
+      <c r="K12" s="15">
+        <f>IF(COUNT(K2:K3,K4:K6,K10:K11)=0,"",SUM(K10:K11))</f>
         <v>4.27</v>
       </c>
-      <c r="I12" s="15">
-        <f>SUMIF($B$2:$B$200,"Debt service",I$2:I$200)</f>
+      <c r="L12" s="15">
+        <f>IF(COUNT(L2:L3,L4:L6,L10:L11)=0,"",SUM(L10:L11))</f>
         <v>4.28</v>
+      </c>
+      <c r="M12" s="15">
+        <f>IF(COUNT(M2:M3,M4:M6,M10:M11)=0,"",SUM(M10:M11))</f>
+        <v>4.29</v>
+      </c>
+      <c r="N12" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N6,N10:N11)=0,"",SUM(N10:N11))</f>
+        <v/>
+      </c>
+      <c r="O12" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O6,O10:O11)=0,"",SUM(O10:O11))</f>
+        <v/>
+      </c>
+      <c r="P12" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P6,P10:P11)=0,"",SUM(P10:P11))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q6,Q10:Q11)=0,"",SUM(Q10:Q11))</f>
+        <v/>
+      </c>
+      <c r="R12" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R6,R10:R11)=0,"",SUM(R10:R11))</f>
+        <v/>
       </c>
     </row>
     <row r="13"/>
@@ -2983,33 +3225,69 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="16" t="str">
         <f>IFERROR(C8/C12,"")</f>
-        <v>0.668213</v>
-      </c>
-      <c r="D14" s="16">
+        <v/>
+      </c>
+      <c r="D14" s="16" t="str">
         <f>IFERROR(D8/D12,"")</f>
-        <v>0.728972</v>
-      </c>
-      <c r="E14" s="16">
+        <v/>
+      </c>
+      <c r="E14" s="16" t="str">
         <f>IFERROR(E8/E12,"")</f>
-        <v>1.72028</v>
+        <v/>
       </c>
       <c r="F14" s="16">
         <f>IFERROR(F8/F12,"")</f>
-        <v>1.812646</v>
+        <v>0.668213</v>
       </c>
       <c r="G14" s="16">
         <f>IFERROR(G8/G12,"")</f>
-        <v>0.791569</v>
+        <v>0.728972</v>
       </c>
       <c r="H14" s="16">
         <f>IFERROR(H8/H12,"")</f>
-        <v>0.805621</v>
+        <v>1.72028</v>
       </c>
       <c r="I14" s="16">
         <f>IFERROR(I8/I12,"")</f>
+        <v>1.812646</v>
+      </c>
+      <c r="J14" s="16">
+        <f>IFERROR(J8/J12,"")</f>
+        <v>0.791569</v>
+      </c>
+      <c r="K14" s="16">
+        <f>IFERROR(K8/K12,"")</f>
+        <v>0.805621</v>
+      </c>
+      <c r="L14" s="16">
+        <f>IFERROR(L8/L12,"")</f>
         <v>1.817757</v>
+      </c>
+      <c r="M14" s="16">
+        <f>IFERROR(M8/M12,"")</f>
+        <v>1.871795</v>
+      </c>
+      <c r="N14" s="16" t="str">
+        <f>IFERROR(N8/N12,"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="16" t="str">
+        <f>IFERROR(O8/O12,"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="16" t="str">
+        <f>IFERROR(P8/P12,"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="16" t="str">
+        <f>IFERROR(Q8/Q12,"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="16" t="str">
+        <f>IFERROR(R8/R12,"")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3035,21 +3313,57 @@
         <f>""</f>
         <v/>
       </c>
-      <c r="F15" s="16">
-        <f>IFERROR(SUM(C8:F8)/SUM(C12:F12),"")</f>
+      <c r="F15" s="16" t="str">
+        <f>IF(COUNT(C8:F8)&lt;4,"",IFERROR(SUM(C8:F8)/SUM(C12:F12),""))</f>
+        <v/>
+      </c>
+      <c r="G15" s="16" t="str">
+        <f>IF(COUNT(D8:G8)&lt;4,"",IFERROR(SUM(D8:G8)/SUM(D12:G12),""))</f>
+        <v/>
+      </c>
+      <c r="H15" s="16" t="str">
+        <f>IF(COUNT(E8:H8)&lt;4,"",IFERROR(SUM(E8:H8)/SUM(E12:H12),""))</f>
+        <v/>
+      </c>
+      <c r="I15" s="16">
+        <f>IF(COUNT(F8:I8)&lt;4,"",IFERROR(SUM(F8:I8)/SUM(F12:I12),""))</f>
         <v>1.231487</v>
       </c>
-      <c r="G15" s="16">
-        <f>IFERROR(SUM(D8:G8)/SUM(D12:G12),"")</f>
+      <c r="J15" s="16">
+        <f>IF(COUNT(G8:J8)&lt;4,"",IFERROR(SUM(G8:J8)/SUM(G12:J12),""))</f>
         <v>1.263589</v>
       </c>
-      <c r="H15" s="16">
-        <f>IFERROR(SUM(E8:H8)/SUM(E12:H12),"")</f>
+      <c r="K15" s="16">
+        <f>IF(COUNT(H8:K8)&lt;4,"",IFERROR(SUM(H8:K8)/SUM(H12:K12),""))</f>
         <v>1.283041</v>
       </c>
-      <c r="I15" s="16">
-        <f>IFERROR(SUM(F8:I8)/SUM(F12:I12),"")</f>
+      <c r="L15" s="16">
+        <f>IF(COUNT(I8:L8)&lt;4,"",IFERROR(SUM(I8:L8)/SUM(I12:L12),""))</f>
         <v>1.307197</v>
+      </c>
+      <c r="M15" s="16">
+        <f>IF(COUNT(J8:M8)&lt;4,"",IFERROR(SUM(J8:M8)/SUM(J12:M12),""))</f>
+        <v>1.322618</v>
+      </c>
+      <c r="N15" s="16" t="str">
+        <f>IF(COUNT(K8:N8)&lt;4,"",IFERROR(SUM(K8:N8)/SUM(K12:N12),""))</f>
+        <v/>
+      </c>
+      <c r="O15" s="16" t="str">
+        <f>IF(COUNT(L8:O8)&lt;4,"",IFERROR(SUM(L8:O8)/SUM(L12:O12),""))</f>
+        <v/>
+      </c>
+      <c r="P15" s="16" t="str">
+        <f>IF(COUNT(M8:P8)&lt;4,"",IFERROR(SUM(M8:P8)/SUM(M12:P12),""))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="16" t="str">
+        <f>IF(COUNT(N8:Q8)&lt;4,"",IFERROR(SUM(N8:Q8)/SUM(N12:Q12),""))</f>
+        <v/>
+      </c>
+      <c r="R15" s="16" t="str">
+        <f>IF(COUNT(O8:R8)&lt;4,"",IFERROR(SUM(O8:R8)/SUM(O12:R12),""))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dashboard builder: one combined coverage chart on page 2, last 8 quarters
- The separate CFADS and DSCR charts become one chart with two stacked
  sections on a shared quarter axis: LTM DSCR with the distribution
  lock-up and default lines on top, CFADS beside stacked debt service
  below.  No dual y-axis; quarterly DSCR bars removed from the chart.
- Covenant lines are unlabeled on the plot; the legend names them with
  their levels.
- Quarters shown defaults to 8 (up to 12), as far as data allows.  The
  examples carry history back to Q1 2024.
- Layout: chart beside the reserves and notes box; cash flow table at
  full width below, tightening when more than 8 quarters are shown.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -1579,11 +1579,11 @@
         </is>
       </c>
       <c r="B27" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">How many of the most recent quarters page 2 shows (1-8).  Enter 3 extra older quarters to show an LTM DSCR for every quarter shown.</t>
+          <t xml:space="preserve">How many of the most recent quarters page 2 shows (1-12), as far as the Debt Service tab has data.  LTM DSCR needs the 3 quarters before each one.</t>
         </is>
       </c>
     </row>
@@ -2730,9 +2730,15 @@
           <t xml:space="preserve">Revenue</t>
         </is>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
+      <c r="C2" s="10">
+        <v>5.42</v>
+      </c>
+      <c r="D2" s="10">
+        <v>9.78</v>
+      </c>
+      <c r="E2" s="10">
+        <v>10.21</v>
+      </c>
       <c r="F2" s="10">
         <v>5.31</v>
       </c>
@@ -2775,9 +2781,15 @@
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
+      <c r="C4" s="10">
+        <v>1.85</v>
+      </c>
+      <c r="D4" s="10">
+        <v>1.95</v>
+      </c>
+      <c r="E4" s="10">
+        <v>2.05</v>
+      </c>
       <c r="F4" s="10">
         <v>1.92</v>
       </c>
@@ -2819,9 +2831,15 @@
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
+      <c r="C5" s="10">
+        <v>0.38</v>
+      </c>
+      <c r="D5" s="10">
+        <v>0.38</v>
+      </c>
+      <c r="E5" s="10">
+        <v>0.38</v>
+      </c>
       <c r="F5" s="10">
         <v>0.4</v>
       </c>
@@ -2863,9 +2881,15 @@
           <t xml:space="preserve">Expense</t>
         </is>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
+      <c r="C6" s="10">
+        <v>0.1</v>
+      </c>
+      <c r="D6" s="10">
+        <v>0.17</v>
+      </c>
+      <c r="E6" s="10">
+        <v>0.2</v>
+      </c>
       <c r="F6" s="10">
         <v>0.11</v>
       </c>
@@ -2907,17 +2931,17 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C7" s="15" t="str">
+      <c r="C7" s="15">
         <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C4:C6))</f>
-        <v/>
-      </c>
-      <c r="D7" s="15" t="str">
+        <v>2.33</v>
+      </c>
+      <c r="D7" s="15">
         <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D4:D6))</f>
-        <v/>
-      </c>
-      <c r="E7" s="15" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="E7" s="15">
         <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E4:E6))</f>
-        <v/>
+        <v>2.63</v>
       </c>
       <c r="F7" s="15">
         <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F4:F6))</f>
@@ -2983,17 +3007,17 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C8" s="15" t="str">
+      <c r="C8" s="15">
         <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C2:C3)-C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="15" t="str">
+        <v>3.09</v>
+      </c>
+      <c r="D8" s="15">
         <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D2:D3)-D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="15" t="str">
+        <v>7.28</v>
+      </c>
+      <c r="E8" s="15">
         <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E2:E3)-E7)</f>
-        <v/>
+        <v>7.58</v>
       </c>
       <c r="F8" s="15">
         <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F2:F3)-F7)</f>
@@ -3060,9 +3084,15 @@
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+      <c r="C10" s="10">
+        <v>2.3</v>
+      </c>
+      <c r="D10" s="10">
+        <v>2.33</v>
+      </c>
+      <c r="E10" s="10">
+        <v>2.37</v>
+      </c>
       <c r="F10" s="10">
         <v>2.4</v>
       </c>
@@ -3104,9 +3134,15 @@
           <t xml:space="preserve">Debt service</t>
         </is>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
+      <c r="C11" s="10">
+        <v>2.05</v>
+      </c>
+      <c r="D11" s="10">
+        <v>2</v>
+      </c>
+      <c r="E11" s="10">
+        <v>1.95</v>
+      </c>
       <c r="F11" s="10">
         <v>1.91</v>
       </c>
@@ -3148,17 +3184,17 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C12" s="15" t="str">
+      <c r="C12" s="15">
         <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C10:C11))</f>
-        <v/>
-      </c>
-      <c r="D12" s="15" t="str">
+        <v>4.35</v>
+      </c>
+      <c r="D12" s="15">
         <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D10:D11))</f>
-        <v/>
-      </c>
-      <c r="E12" s="15" t="str">
+        <v>4.33</v>
+      </c>
+      <c r="E12" s="15">
         <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E10:E11))</f>
-        <v/>
+        <v>4.32</v>
       </c>
       <c r="F12" s="15">
         <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F10:F11))</f>
@@ -3225,17 +3261,17 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C14" s="16" t="str">
+      <c r="C14" s="16">
         <f>IFERROR(C8/C12,"")</f>
-        <v/>
-      </c>
-      <c r="D14" s="16" t="str">
+        <v>0.710345</v>
+      </c>
+      <c r="D14" s="16">
         <f>IFERROR(D8/D12,"")</f>
-        <v/>
-      </c>
-      <c r="E14" s="16" t="str">
+        <v>1.681293</v>
+      </c>
+      <c r="E14" s="16">
         <f>IFERROR(E8/E12,"")</f>
-        <v/>
+        <v>1.75463</v>
       </c>
       <c r="F14" s="16">
         <f>IFERROR(F8/F12,"")</f>
@@ -3313,17 +3349,17 @@
         <f>""</f>
         <v/>
       </c>
-      <c r="F15" s="16" t="str">
+      <c r="F15" s="16">
         <f>IF(COUNT(C8:F8)&lt;4,"",IFERROR(SUM(C8:F8)/SUM(C12:F12),""))</f>
-        <v/>
-      </c>
-      <c r="G15" s="16" t="str">
+        <v>1.203351</v>
+      </c>
+      <c r="G15" s="16">
         <f>IF(COUNT(D8:G8)&lt;4,"",IFERROR(SUM(D8:G8)/SUM(D12:G12),""))</f>
-        <v/>
-      </c>
-      <c r="H15" s="16" t="str">
+        <v>1.209977</v>
+      </c>
+      <c r="H15" s="16">
         <f>IF(COUNT(E8:H8)&lt;4,"",IFERROR(SUM(E8:H8)/SUM(E12:H12),""))</f>
-        <v/>
+        <v>1.218605</v>
       </c>
       <c r="I15" s="16">
         <f>IF(COUNT(F8:I8)&lt;4,"",IFERROR(SUM(F8:I8)/SUM(F12:I12),""))</f>

</xml_diff>

<commit_message>
Dashboard builder: one Property and Other Expenses row on the Debt Service tab
The example workbooks combine Property taxes and Other taxes into a
single Expense row, Property and Other Expenses (the old rows summed);
CFADS and DSCR are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -2823,7 +2823,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Property taxes</t>
+          <t xml:space="preserve">Property and Other Expenses</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -2832,37 +2832,37 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <v>0.38</v>
+        <v>0.48</v>
       </c>
       <c r="D5" s="10">
-        <v>0.38</v>
+        <v>0.55</v>
       </c>
       <c r="E5" s="10">
-        <v>0.38</v>
+        <v>0.58</v>
       </c>
       <c r="F5" s="10">
-        <v>0.4</v>
+        <v>0.51</v>
       </c>
       <c r="G5" s="10">
-        <v>0.4</v>
+        <v>0.49</v>
       </c>
       <c r="H5" s="10">
-        <v>0.4</v>
+        <v>0.58</v>
       </c>
       <c r="I5" s="10">
-        <v>0.4</v>
+        <v>0.61</v>
       </c>
       <c r="J5" s="10">
-        <v>0.42</v>
+        <v>0.52</v>
       </c>
       <c r="K5" s="10">
-        <v>0.45</v>
+        <v>0.53</v>
       </c>
       <c r="L5" s="10">
-        <v>0.45</v>
+        <v>0.64</v>
       </c>
       <c r="M5" s="10">
-        <v>0.45</v>
+        <v>0.67</v>
       </c>
       <c r="N5" s="10"/>
       <c r="O5" s="10"/>
@@ -2871,59 +2871,85 @@
       <c r="R5" s="10"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Other taxes</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Expense</t>
-        </is>
-      </c>
-      <c r="C6" s="10">
-        <v>0.1</v>
-      </c>
-      <c r="D6" s="10">
-        <v>0.17</v>
-      </c>
-      <c r="E6" s="10">
-        <v>0.2</v>
-      </c>
-      <c r="F6" s="10">
-        <v>0.11</v>
-      </c>
-      <c r="G6" s="10">
-        <v>0.09</v>
-      </c>
-      <c r="H6" s="10">
-        <v>0.18</v>
-      </c>
-      <c r="I6" s="10">
-        <v>0.21</v>
-      </c>
-      <c r="J6" s="10">
-        <v>0.1</v>
-      </c>
-      <c r="K6" s="10">
-        <v>0.08</v>
-      </c>
-      <c r="L6" s="10">
-        <v>0.19</v>
-      </c>
-      <c r="M6" s="10">
-        <v>0.22</v>
-      </c>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total O&amp;M costs</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C6" s="15">
+        <f>IF(COUNT(C2:C3,C4:C5,C9:C10)=0,"",SUM(C4:C5))</f>
+        <v>2.33</v>
+      </c>
+      <c r="D6" s="15">
+        <f>IF(COUNT(D2:D3,D4:D5,D9:D10)=0,"",SUM(D4:D5))</f>
+        <v>2.5</v>
+      </c>
+      <c r="E6" s="15">
+        <f>IF(COUNT(E2:E3,E4:E5,E9:E10)=0,"",SUM(E4:E5))</f>
+        <v>2.63</v>
+      </c>
+      <c r="F6" s="15">
+        <f>IF(COUNT(F2:F3,F4:F5,F9:F10)=0,"",SUM(F4:F5))</f>
+        <v>2.43</v>
+      </c>
+      <c r="G6" s="15">
+        <f>IF(COUNT(G2:G3,G4:G5,G9:G10)=0,"",SUM(G4:G5))</f>
+        <v>2.5</v>
+      </c>
+      <c r="H6" s="15">
+        <f>IF(COUNT(H2:H3,H4:H5,H9:H10)=0,"",SUM(H4:H5))</f>
+        <v>2.66</v>
+      </c>
+      <c r="I6" s="15">
+        <f>IF(COUNT(I2:I3,I4:I5,I9:I10)=0,"",SUM(I4:I5))</f>
+        <v>2.78</v>
+      </c>
+      <c r="J6" s="15">
+        <f>IF(COUNT(J2:J3,J4:J5,J9:J10)=0,"",SUM(J4:J5))</f>
+        <v>2.55</v>
+      </c>
+      <c r="K6" s="15">
+        <f>IF(COUNT(K2:K3,K4:K5,K9:K10)=0,"",SUM(K4:K5))</f>
+        <v>2.64</v>
+      </c>
+      <c r="L6" s="15">
+        <f>IF(COUNT(L2:L3,L4:L5,L9:L10)=0,"",SUM(L4:L5))</f>
+        <v>2.83</v>
+      </c>
+      <c r="M6" s="15">
+        <f>IF(COUNT(M2:M3,M4:M5,M9:M10)=0,"",SUM(M4:M5))</f>
+        <v>2.91</v>
+      </c>
+      <c r="N6" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N5,N9:N10)=0,"",SUM(N4:N5))</f>
+        <v/>
+      </c>
+      <c r="O6" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O5,O9:O10)=0,"",SUM(O4:O5))</f>
+        <v/>
+      </c>
+      <c r="P6" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P5,P9:P10)=0,"",SUM(P4:P5))</f>
+        <v/>
+      </c>
+      <c r="Q6" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q10)=0,"",SUM(Q4:Q5))</f>
+        <v/>
+      </c>
+      <c r="R6" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R5,R9:R10)=0,"",SUM(R4:R5))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total O&amp;M costs</t>
+          <t xml:space="preserve">CFADS</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -2932,151 +2958,125 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C4:C6))</f>
+        <f>IF(COUNT(C2:C3,C4:C5,C9:C10)=0,"",SUM(C2:C3)-C6)</f>
+        <v>3.09</v>
+      </c>
+      <c r="D7" s="15">
+        <f>IF(COUNT(D2:D3,D4:D5,D9:D10)=0,"",SUM(D2:D3)-D6)</f>
+        <v>7.28</v>
+      </c>
+      <c r="E7" s="15">
+        <f>IF(COUNT(E2:E3,E4:E5,E9:E10)=0,"",SUM(E2:E3)-E6)</f>
+        <v>7.58</v>
+      </c>
+      <c r="F7" s="15">
+        <f>IF(COUNT(F2:F3,F4:F5,F9:F10)=0,"",SUM(F2:F3)-F6)</f>
+        <v>2.88</v>
+      </c>
+      <c r="G7" s="15">
+        <f>IF(COUNT(G2:G3,G4:G5,G9:G10)=0,"",SUM(G2:G3)-G6)</f>
+        <v>3.12</v>
+      </c>
+      <c r="H7" s="15">
+        <f>IF(COUNT(H2:H3,H4:H5,H9:H10)=0,"",SUM(H2:H3)-H6)</f>
+        <v>7.38</v>
+      </c>
+      <c r="I7" s="15">
+        <f>IF(COUNT(I2:I3,I4:I5,I9:I10)=0,"",SUM(I2:I3)-I6)</f>
+        <v>7.74</v>
+      </c>
+      <c r="J7" s="15">
+        <f>IF(COUNT(J2:J3,J4:J5,J9:J10)=0,"",SUM(J2:J3)-J6)</f>
+        <v>3.38</v>
+      </c>
+      <c r="K7" s="15">
+        <f>IF(COUNT(K2:K3,K4:K5,K9:K10)=0,"",SUM(K2:K3)-K6)</f>
+        <v>3.44</v>
+      </c>
+      <c r="L7" s="15">
+        <f>IF(COUNT(L2:L3,L4:L5,L9:L10)=0,"",SUM(L2:L3)-L6)</f>
+        <v>7.78</v>
+      </c>
+      <c r="M7" s="15">
+        <f>IF(COUNT(M2:M3,M4:M5,M9:M10)=0,"",SUM(M2:M3)-M6)</f>
+        <v>8.03</v>
+      </c>
+      <c r="N7" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N5,N9:N10)=0,"",SUM(N2:N3)-N6)</f>
+        <v/>
+      </c>
+      <c r="O7" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O5,O9:O10)=0,"",SUM(O2:O3)-O6)</f>
+        <v/>
+      </c>
+      <c r="P7" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P5,P9:P10)=0,"",SUM(P2:P3)-P6)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q10)=0,"",SUM(Q2:Q3)-Q6)</f>
+        <v/>
+      </c>
+      <c r="R7" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R5,R9:R10)=0,"",SUM(R2:R3)-R6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Principal</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service</t>
+        </is>
+      </c>
+      <c r="C9" s="10">
+        <v>2.3</v>
+      </c>
+      <c r="D9" s="10">
         <v>2.33</v>
       </c>
-      <c r="D7" s="15">
-        <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D4:D6))</f>
-        <v>2.5</v>
-      </c>
-      <c r="E7" s="15">
-        <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E4:E6))</f>
-        <v>2.63</v>
-      </c>
-      <c r="F7" s="15">
-        <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F4:F6))</f>
-        <v>2.43</v>
-      </c>
-      <c r="G7" s="15">
-        <f>IF(COUNT(G2:G3,G4:G6,G10:G11)=0,"",SUM(G4:G6))</f>
-        <v>2.5</v>
-      </c>
-      <c r="H7" s="15">
-        <f>IF(COUNT(H2:H3,H4:H6,H10:H11)=0,"",SUM(H4:H6))</f>
-        <v>2.66</v>
-      </c>
-      <c r="I7" s="15">
-        <f>IF(COUNT(I2:I3,I4:I6,I10:I11)=0,"",SUM(I4:I6))</f>
-        <v>2.78</v>
-      </c>
-      <c r="J7" s="15">
-        <f>IF(COUNT(J2:J3,J4:J6,J10:J11)=0,"",SUM(J4:J6))</f>
-        <v>2.55</v>
-      </c>
-      <c r="K7" s="15">
-        <f>IF(COUNT(K2:K3,K4:K6,K10:K11)=0,"",SUM(K4:K6))</f>
-        <v>2.64</v>
-      </c>
-      <c r="L7" s="15">
-        <f>IF(COUNT(L2:L3,L4:L6,L10:L11)=0,"",SUM(L4:L6))</f>
-        <v>2.83</v>
-      </c>
-      <c r="M7" s="15">
-        <f>IF(COUNT(M2:M3,M4:M6,M10:M11)=0,"",SUM(M4:M6))</f>
-        <v>2.91</v>
-      </c>
-      <c r="N7" s="15" t="str">
-        <f>IF(COUNT(N2:N3,N4:N6,N10:N11)=0,"",SUM(N4:N6))</f>
-        <v/>
-      </c>
-      <c r="O7" s="15" t="str">
-        <f>IF(COUNT(O2:O3,O4:O6,O10:O11)=0,"",SUM(O4:O6))</f>
-        <v/>
-      </c>
-      <c r="P7" s="15" t="str">
-        <f>IF(COUNT(P2:P3,P4:P6,P10:P11)=0,"",SUM(P4:P6))</f>
-        <v/>
-      </c>
-      <c r="Q7" s="15" t="str">
-        <f>IF(COUNT(Q2:Q3,Q4:Q6,Q10:Q11)=0,"",SUM(Q4:Q6))</f>
-        <v/>
-      </c>
-      <c r="R7" s="15" t="str">
-        <f>IF(COUNT(R2:R3,R4:R6,R10:R11)=0,"",SUM(R4:R6))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CFADS</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Calculated</t>
-        </is>
-      </c>
-      <c r="C8" s="15">
-        <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C2:C3)-C7)</f>
-        <v>3.09</v>
-      </c>
-      <c r="D8" s="15">
-        <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D2:D3)-D7)</f>
-        <v>7.28</v>
-      </c>
-      <c r="E8" s="15">
-        <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E2:E3)-E7)</f>
-        <v>7.58</v>
-      </c>
-      <c r="F8" s="15">
-        <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F2:F3)-F7)</f>
-        <v>2.88</v>
-      </c>
-      <c r="G8" s="15">
-        <f>IF(COUNT(G2:G3,G4:G6,G10:G11)=0,"",SUM(G2:G3)-G7)</f>
-        <v>3.12</v>
-      </c>
-      <c r="H8" s="15">
-        <f>IF(COUNT(H2:H3,H4:H6,H10:H11)=0,"",SUM(H2:H3)-H7)</f>
-        <v>7.38</v>
-      </c>
-      <c r="I8" s="15">
-        <f>IF(COUNT(I2:I3,I4:I6,I10:I11)=0,"",SUM(I2:I3)-I7)</f>
-        <v>7.74</v>
-      </c>
-      <c r="J8" s="15">
-        <f>IF(COUNT(J2:J3,J4:J6,J10:J11)=0,"",SUM(J2:J3)-J7)</f>
-        <v>3.38</v>
-      </c>
-      <c r="K8" s="15">
-        <f>IF(COUNT(K2:K3,K4:K6,K10:K11)=0,"",SUM(K2:K3)-K7)</f>
-        <v>3.44</v>
-      </c>
-      <c r="L8" s="15">
-        <f>IF(COUNT(L2:L3,L4:L6,L10:L11)=0,"",SUM(L2:L3)-L7)</f>
-        <v>7.78</v>
-      </c>
-      <c r="M8" s="15">
-        <f>IF(COUNT(M2:M3,M4:M6,M10:M11)=0,"",SUM(M2:M3)-M7)</f>
-        <v>8.03</v>
-      </c>
-      <c r="N8" s="15" t="str">
-        <f>IF(COUNT(N2:N3,N4:N6,N10:N11)=0,"",SUM(N2:N3)-N7)</f>
-        <v/>
-      </c>
-      <c r="O8" s="15" t="str">
-        <f>IF(COUNT(O2:O3,O4:O6,O10:O11)=0,"",SUM(O2:O3)-O7)</f>
-        <v/>
-      </c>
-      <c r="P8" s="15" t="str">
-        <f>IF(COUNT(P2:P3,P4:P6,P10:P11)=0,"",SUM(P2:P3)-P7)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="15" t="str">
-        <f>IF(COUNT(Q2:Q3,Q4:Q6,Q10:Q11)=0,"",SUM(Q2:Q3)-Q7)</f>
-        <v/>
-      </c>
-      <c r="R8" s="15" t="str">
-        <f>IF(COUNT(R2:R3,R4:R6,R10:R11)=0,"",SUM(R2:R3)-R7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9"/>
+      <c r="E9" s="10">
+        <v>2.37</v>
+      </c>
+      <c r="F9" s="10">
+        <v>2.4</v>
+      </c>
+      <c r="G9" s="10">
+        <v>2.42</v>
+      </c>
+      <c r="H9" s="10">
+        <v>2.48</v>
+      </c>
+      <c r="I9" s="10">
+        <v>2.51</v>
+      </c>
+      <c r="J9" s="10">
+        <v>2.57</v>
+      </c>
+      <c r="K9" s="10">
+        <v>2.62</v>
+      </c>
+      <c r="L9" s="10">
+        <v>2.68</v>
+      </c>
+      <c r="M9" s="10">
+        <v>2.74</v>
+      </c>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+    </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Principal</t>
+          <t xml:space="preserve">Interest</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -3085,37 +3085,37 @@
         </is>
       </c>
       <c r="C10" s="10">
-        <v>2.3</v>
+        <v>2.05</v>
       </c>
       <c r="D10" s="10">
-        <v>2.33</v>
+        <v>2</v>
       </c>
       <c r="E10" s="10">
-        <v>2.37</v>
+        <v>1.95</v>
       </c>
       <c r="F10" s="10">
-        <v>2.4</v>
+        <v>1.91</v>
       </c>
       <c r="G10" s="10">
-        <v>2.42</v>
+        <v>1.86</v>
       </c>
       <c r="H10" s="10">
-        <v>2.48</v>
+        <v>1.81</v>
       </c>
       <c r="I10" s="10">
-        <v>2.51</v>
+        <v>1.76</v>
       </c>
       <c r="J10" s="10">
-        <v>2.57</v>
+        <v>1.7</v>
       </c>
       <c r="K10" s="10">
-        <v>2.62</v>
+        <v>1.65</v>
       </c>
       <c r="L10" s="10">
-        <v>2.68</v>
+        <v>1.6</v>
       </c>
       <c r="M10" s="10">
-        <v>2.74</v>
+        <v>1.55</v>
       </c>
       <c r="N10" s="10"/>
       <c r="O10" s="10"/>
@@ -3124,136 +3124,162 @@
       <c r="R10" s="10"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interest</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Debt service</t>
-        </is>
-      </c>
-      <c r="C11" s="10">
-        <v>2.05</v>
-      </c>
-      <c r="D11" s="10">
-        <v>2</v>
-      </c>
-      <c r="E11" s="10">
-        <v>1.95</v>
-      </c>
-      <c r="F11" s="10">
-        <v>1.91</v>
-      </c>
-      <c r="G11" s="10">
-        <v>1.86</v>
-      </c>
-      <c r="H11" s="10">
-        <v>1.81</v>
-      </c>
-      <c r="I11" s="10">
-        <v>1.76</v>
-      </c>
-      <c r="J11" s="10">
-        <v>1.7</v>
-      </c>
-      <c r="K11" s="10">
-        <v>1.65</v>
-      </c>
-      <c r="L11" s="10">
-        <v>1.6</v>
-      </c>
-      <c r="M11" s="10">
-        <v>1.55</v>
-      </c>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="10"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Total debt service costs</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C12" s="15">
-        <f>IF(COUNT(C2:C3,C4:C6,C10:C11)=0,"",SUM(C10:C11))</f>
+      <c r="C11" s="15">
+        <f>IF(COUNT(C2:C3,C4:C5,C9:C10)=0,"",SUM(C9:C10))</f>
         <v>4.35</v>
       </c>
-      <c r="D12" s="15">
-        <f>IF(COUNT(D2:D3,D4:D6,D10:D11)=0,"",SUM(D10:D11))</f>
+      <c r="D11" s="15">
+        <f>IF(COUNT(D2:D3,D4:D5,D9:D10)=0,"",SUM(D9:D10))</f>
         <v>4.33</v>
       </c>
-      <c r="E12" s="15">
-        <f>IF(COUNT(E2:E3,E4:E6,E10:E11)=0,"",SUM(E10:E11))</f>
+      <c r="E11" s="15">
+        <f>IF(COUNT(E2:E3,E4:E5,E9:E10)=0,"",SUM(E9:E10))</f>
         <v>4.32</v>
       </c>
-      <c r="F12" s="15">
-        <f>IF(COUNT(F2:F3,F4:F6,F10:F11)=0,"",SUM(F10:F11))</f>
+      <c r="F11" s="15">
+        <f>IF(COUNT(F2:F3,F4:F5,F9:F10)=0,"",SUM(F9:F10))</f>
         <v>4.31</v>
       </c>
-      <c r="G12" s="15">
-        <f>IF(COUNT(G2:G3,G4:G6,G10:G11)=0,"",SUM(G10:G11))</f>
+      <c r="G11" s="15">
+        <f>IF(COUNT(G2:G3,G4:G5,G9:G10)=0,"",SUM(G9:G10))</f>
         <v>4.28</v>
       </c>
-      <c r="H12" s="15">
-        <f>IF(COUNT(H2:H3,H4:H6,H10:H11)=0,"",SUM(H10:H11))</f>
+      <c r="H11" s="15">
+        <f>IF(COUNT(H2:H3,H4:H5,H9:H10)=0,"",SUM(H9:H10))</f>
         <v>4.29</v>
       </c>
-      <c r="I12" s="15">
-        <f>IF(COUNT(I2:I3,I4:I6,I10:I11)=0,"",SUM(I10:I11))</f>
+      <c r="I11" s="15">
+        <f>IF(COUNT(I2:I3,I4:I5,I9:I10)=0,"",SUM(I9:I10))</f>
         <v>4.27</v>
       </c>
-      <c r="J12" s="15">
-        <f>IF(COUNT(J2:J3,J4:J6,J10:J11)=0,"",SUM(J10:J11))</f>
+      <c r="J11" s="15">
+        <f>IF(COUNT(J2:J3,J4:J5,J9:J10)=0,"",SUM(J9:J10))</f>
         <v>4.27</v>
       </c>
-      <c r="K12" s="15">
-        <f>IF(COUNT(K2:K3,K4:K6,K10:K11)=0,"",SUM(K10:K11))</f>
+      <c r="K11" s="15">
+        <f>IF(COUNT(K2:K3,K4:K5,K9:K10)=0,"",SUM(K9:K10))</f>
         <v>4.27</v>
       </c>
-      <c r="L12" s="15">
-        <f>IF(COUNT(L2:L3,L4:L6,L10:L11)=0,"",SUM(L10:L11))</f>
+      <c r="L11" s="15">
+        <f>IF(COUNT(L2:L3,L4:L5,L9:L10)=0,"",SUM(L9:L10))</f>
         <v>4.28</v>
       </c>
-      <c r="M12" s="15">
-        <f>IF(COUNT(M2:M3,M4:M6,M10:M11)=0,"",SUM(M10:M11))</f>
+      <c r="M11" s="15">
+        <f>IF(COUNT(M2:M3,M4:M5,M9:M10)=0,"",SUM(M9:M10))</f>
         <v>4.29</v>
       </c>
-      <c r="N12" s="15" t="str">
-        <f>IF(COUNT(N2:N3,N4:N6,N10:N11)=0,"",SUM(N10:N11))</f>
-        <v/>
-      </c>
-      <c r="O12" s="15" t="str">
-        <f>IF(COUNT(O2:O3,O4:O6,O10:O11)=0,"",SUM(O10:O11))</f>
-        <v/>
-      </c>
-      <c r="P12" s="15" t="str">
-        <f>IF(COUNT(P2:P3,P4:P6,P10:P11)=0,"",SUM(P10:P11))</f>
-        <v/>
-      </c>
-      <c r="Q12" s="15" t="str">
-        <f>IF(COUNT(Q2:Q3,Q4:Q6,Q10:Q11)=0,"",SUM(Q10:Q11))</f>
-        <v/>
-      </c>
-      <c r="R12" s="15" t="str">
-        <f>IF(COUNT(R2:R3,R4:R6,R10:R11)=0,"",SUM(R10:R11))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13"/>
+      <c r="N11" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N5,N9:N10)=0,"",SUM(N9:N10))</f>
+        <v/>
+      </c>
+      <c r="O11" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O5,O9:O10)=0,"",SUM(O9:O10))</f>
+        <v/>
+      </c>
+      <c r="P11" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P5,P9:P10)=0,"",SUM(P9:P10))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q10)=0,"",SUM(Q9:Q10))</f>
+        <v/>
+      </c>
+      <c r="R11" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R5,R9:R10)=0,"",SUM(R9:R10))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DSCR - quarter</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C13" s="16">
+        <f>IFERROR(C7/C11,"")</f>
+        <v>0.710345</v>
+      </c>
+      <c r="D13" s="16">
+        <f>IFERROR(D7/D11,"")</f>
+        <v>1.681293</v>
+      </c>
+      <c r="E13" s="16">
+        <f>IFERROR(E7/E11,"")</f>
+        <v>1.75463</v>
+      </c>
+      <c r="F13" s="16">
+        <f>IFERROR(F7/F11,"")</f>
+        <v>0.668213</v>
+      </c>
+      <c r="G13" s="16">
+        <f>IFERROR(G7/G11,"")</f>
+        <v>0.728972</v>
+      </c>
+      <c r="H13" s="16">
+        <f>IFERROR(H7/H11,"")</f>
+        <v>1.72028</v>
+      </c>
+      <c r="I13" s="16">
+        <f>IFERROR(I7/I11,"")</f>
+        <v>1.812646</v>
+      </c>
+      <c r="J13" s="16">
+        <f>IFERROR(J7/J11,"")</f>
+        <v>0.791569</v>
+      </c>
+      <c r="K13" s="16">
+        <f>IFERROR(K7/K11,"")</f>
+        <v>0.805621</v>
+      </c>
+      <c r="L13" s="16">
+        <f>IFERROR(L7/L11,"")</f>
+        <v>1.817757</v>
+      </c>
+      <c r="M13" s="16">
+        <f>IFERROR(M7/M11,"")</f>
+        <v>1.871795</v>
+      </c>
+      <c r="N13" s="16" t="str">
+        <f>IFERROR(N7/N11,"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="16" t="str">
+        <f>IFERROR(O7/O11,"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="16" t="str">
+        <f>IFERROR(P7/P11,"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="16" t="str">
+        <f>IFERROR(Q7/Q11,"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="16" t="str">
+        <f>IFERROR(R7/R11,"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSCR - quarter</t>
+          <t xml:space="preserve">DSCR - LTM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -3261,144 +3287,68 @@
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C14" s="16">
-        <f>IFERROR(C8/C12,"")</f>
-        <v>0.710345</v>
-      </c>
-      <c r="D14" s="16">
-        <f>IFERROR(D8/D12,"")</f>
-        <v>1.681293</v>
-      </c>
-      <c r="E14" s="16">
-        <f>IFERROR(E8/E12,"")</f>
-        <v>1.75463</v>
+      <c r="C14" s="16" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="D14" s="16" t="str">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="E14" s="16" t="str">
+        <f>""</f>
+        <v/>
       </c>
       <c r="F14" s="16">
-        <f>IFERROR(F8/F12,"")</f>
-        <v>0.668213</v>
+        <f>IF(COUNT(C7:F7)&lt;4,"",IFERROR(SUM(C7:F7)/SUM(C11:F11),""))</f>
+        <v>1.203351</v>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(G8/G12,"")</f>
-        <v>0.728972</v>
+        <f>IF(COUNT(D7:G7)&lt;4,"",IFERROR(SUM(D7:G7)/SUM(D11:G11),""))</f>
+        <v>1.209977</v>
       </c>
       <c r="H14" s="16">
-        <f>IFERROR(H8/H12,"")</f>
-        <v>1.72028</v>
+        <f>IF(COUNT(E7:H7)&lt;4,"",IFERROR(SUM(E7:H7)/SUM(E11:H11),""))</f>
+        <v>1.218605</v>
       </c>
       <c r="I14" s="16">
-        <f>IFERROR(I8/I12,"")</f>
-        <v>1.812646</v>
+        <f>IF(COUNT(F7:I7)&lt;4,"",IFERROR(SUM(F7:I7)/SUM(F11:I11),""))</f>
+        <v>1.231487</v>
       </c>
       <c r="J14" s="16">
-        <f>IFERROR(J8/J12,"")</f>
-        <v>0.791569</v>
+        <f>IF(COUNT(G7:J7)&lt;4,"",IFERROR(SUM(G7:J7)/SUM(G11:J11),""))</f>
+        <v>1.263589</v>
       </c>
       <c r="K14" s="16">
-        <f>IFERROR(K8/K12,"")</f>
-        <v>0.805621</v>
+        <f>IF(COUNT(H7:K7)&lt;4,"",IFERROR(SUM(H7:K7)/SUM(H11:K11),""))</f>
+        <v>1.283041</v>
       </c>
       <c r="L14" s="16">
-        <f>IFERROR(L8/L12,"")</f>
-        <v>1.817757</v>
+        <f>IF(COUNT(I7:L7)&lt;4,"",IFERROR(SUM(I7:L7)/SUM(I11:L11),""))</f>
+        <v>1.307197</v>
       </c>
       <c r="M14" s="16">
-        <f>IFERROR(M8/M12,"")</f>
-        <v>1.871795</v>
+        <f>IF(COUNT(J7:M7)&lt;4,"",IFERROR(SUM(J7:M7)/SUM(J11:M11),""))</f>
+        <v>1.322618</v>
       </c>
       <c r="N14" s="16" t="str">
-        <f>IFERROR(N8/N12,"")</f>
+        <f>IF(COUNT(K7:N7)&lt;4,"",IFERROR(SUM(K7:N7)/SUM(K11:N11),""))</f>
         <v/>
       </c>
       <c r="O14" s="16" t="str">
-        <f>IFERROR(O8/O12,"")</f>
+        <f>IF(COUNT(L7:O7)&lt;4,"",IFERROR(SUM(L7:O7)/SUM(L11:O11),""))</f>
         <v/>
       </c>
       <c r="P14" s="16" t="str">
-        <f>IFERROR(P8/P12,"")</f>
+        <f>IF(COUNT(M7:P7)&lt;4,"",IFERROR(SUM(M7:P7)/SUM(M11:P11),""))</f>
         <v/>
       </c>
       <c r="Q14" s="16" t="str">
-        <f>IFERROR(Q8/Q12,"")</f>
+        <f>IF(COUNT(N7:Q7)&lt;4,"",IFERROR(SUM(N7:Q7)/SUM(N11:Q11),""))</f>
         <v/>
       </c>
       <c r="R14" s="16" t="str">
-        <f>IFERROR(R8/R12,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DSCR - LTM</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Calculated</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="D15" s="16" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="E15" s="16" t="str">
-        <f>""</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
-        <f>IF(COUNT(C8:F8)&lt;4,"",IFERROR(SUM(C8:F8)/SUM(C12:F12),""))</f>
-        <v>1.203351</v>
-      </c>
-      <c r="G15" s="16">
-        <f>IF(COUNT(D8:G8)&lt;4,"",IFERROR(SUM(D8:G8)/SUM(D12:G12),""))</f>
-        <v>1.209977</v>
-      </c>
-      <c r="H15" s="16">
-        <f>IF(COUNT(E8:H8)&lt;4,"",IFERROR(SUM(E8:H8)/SUM(E12:H12),""))</f>
-        <v>1.218605</v>
-      </c>
-      <c r="I15" s="16">
-        <f>IF(COUNT(F8:I8)&lt;4,"",IFERROR(SUM(F8:I8)/SUM(F12:I12),""))</f>
-        <v>1.231487</v>
-      </c>
-      <c r="J15" s="16">
-        <f>IF(COUNT(G8:J8)&lt;4,"",IFERROR(SUM(G8:J8)/SUM(G12:J12),""))</f>
-        <v>1.263589</v>
-      </c>
-      <c r="K15" s="16">
-        <f>IF(COUNT(H8:K8)&lt;4,"",IFERROR(SUM(H8:K8)/SUM(H12:K12),""))</f>
-        <v>1.283041</v>
-      </c>
-      <c r="L15" s="16">
-        <f>IF(COUNT(I8:L8)&lt;4,"",IFERROR(SUM(I8:L8)/SUM(I12:L12),""))</f>
-        <v>1.307197</v>
-      </c>
-      <c r="M15" s="16">
-        <f>IF(COUNT(J8:M8)&lt;4,"",IFERROR(SUM(J8:M8)/SUM(J12:M12),""))</f>
-        <v>1.322618</v>
-      </c>
-      <c r="N15" s="16" t="str">
-        <f>IF(COUNT(K8:N8)&lt;4,"",IFERROR(SUM(K8:N8)/SUM(K12:N12),""))</f>
-        <v/>
-      </c>
-      <c r="O15" s="16" t="str">
-        <f>IF(COUNT(L8:O8)&lt;4,"",IFERROR(SUM(L8:O8)/SUM(L12:O12),""))</f>
-        <v/>
-      </c>
-      <c r="P15" s="16" t="str">
-        <f>IF(COUNT(M8:P8)&lt;4,"",IFERROR(SUM(M8:P8)/SUM(M12:P12),""))</f>
-        <v/>
-      </c>
-      <c r="Q15" s="16" t="str">
-        <f>IF(COUNT(N8:Q8)&lt;4,"",IFERROR(SUM(N8:Q8)/SUM(N12:Q12),""))</f>
-        <v/>
-      </c>
-      <c r="R15" s="16" t="str">
-        <f>IF(COUNT(O8:R8)&lt;4,"",IFERROR(SUM(O8:R8)/SUM(O12:R12),""))</f>
+        <f>IF(COUNT(O7:R7)&lt;4,"",IFERROR(SUM(O7:R7)/SUM(O11:R11),""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard builder: cash flow decimals default to 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -1658,11 +1658,11 @@
         </is>
       </c>
       <c r="B32" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decimals in the page 2 cash flow table.</t>
+          <t xml:space="preserve">Decimals in the page 2 cash flow table and reserves (default 1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard builder: swap settlements and agency fees; robust extra debt lines
- Examples add Interest rate swap settlements and Agency fees as Debt
  service rows (swap includes net receipts as negatives).
- The page 2 stacked bar shows up to 3 debt lines as-is; with more, the
  first two plus one Other debt service piece.  A net negative piece
  (e.g. a swap receipt) reduces the piece below it, so each bar always
  equals total debt service.  The table still lists every line.
- Fix: a fourth debt line no longer reuses the first line's color.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -2882,67 +2882,67 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>IF(COUNT(C2:C3,C4:C5,C9:C10)=0,"",SUM(C4:C5))</f>
+        <f>IF(COUNT(C2:C3,C4:C5,C9:C12)=0,"",SUM(C4:C5))</f>
         <v>2.33</v>
       </c>
       <c r="D6" s="15">
-        <f>IF(COUNT(D2:D3,D4:D5,D9:D10)=0,"",SUM(D4:D5))</f>
+        <f>IF(COUNT(D2:D3,D4:D5,D9:D12)=0,"",SUM(D4:D5))</f>
         <v>2.5</v>
       </c>
       <c r="E6" s="15">
-        <f>IF(COUNT(E2:E3,E4:E5,E9:E10)=0,"",SUM(E4:E5))</f>
+        <f>IF(COUNT(E2:E3,E4:E5,E9:E12)=0,"",SUM(E4:E5))</f>
         <v>2.63</v>
       </c>
       <c r="F6" s="15">
-        <f>IF(COUNT(F2:F3,F4:F5,F9:F10)=0,"",SUM(F4:F5))</f>
+        <f>IF(COUNT(F2:F3,F4:F5,F9:F12)=0,"",SUM(F4:F5))</f>
         <v>2.43</v>
       </c>
       <c r="G6" s="15">
-        <f>IF(COUNT(G2:G3,G4:G5,G9:G10)=0,"",SUM(G4:G5))</f>
+        <f>IF(COUNT(G2:G3,G4:G5,G9:G12)=0,"",SUM(G4:G5))</f>
         <v>2.5</v>
       </c>
       <c r="H6" s="15">
-        <f>IF(COUNT(H2:H3,H4:H5,H9:H10)=0,"",SUM(H4:H5))</f>
+        <f>IF(COUNT(H2:H3,H4:H5,H9:H12)=0,"",SUM(H4:H5))</f>
         <v>2.66</v>
       </c>
       <c r="I6" s="15">
-        <f>IF(COUNT(I2:I3,I4:I5,I9:I10)=0,"",SUM(I4:I5))</f>
+        <f>IF(COUNT(I2:I3,I4:I5,I9:I12)=0,"",SUM(I4:I5))</f>
         <v>2.78</v>
       </c>
       <c r="J6" s="15">
-        <f>IF(COUNT(J2:J3,J4:J5,J9:J10)=0,"",SUM(J4:J5))</f>
+        <f>IF(COUNT(J2:J3,J4:J5,J9:J12)=0,"",SUM(J4:J5))</f>
         <v>2.55</v>
       </c>
       <c r="K6" s="15">
-        <f>IF(COUNT(K2:K3,K4:K5,K9:K10)=0,"",SUM(K4:K5))</f>
+        <f>IF(COUNT(K2:K3,K4:K5,K9:K12)=0,"",SUM(K4:K5))</f>
         <v>2.64</v>
       </c>
       <c r="L6" s="15">
-        <f>IF(COUNT(L2:L3,L4:L5,L9:L10)=0,"",SUM(L4:L5))</f>
+        <f>IF(COUNT(L2:L3,L4:L5,L9:L12)=0,"",SUM(L4:L5))</f>
         <v>2.83</v>
       </c>
       <c r="M6" s="15">
-        <f>IF(COUNT(M2:M3,M4:M5,M9:M10)=0,"",SUM(M4:M5))</f>
+        <f>IF(COUNT(M2:M3,M4:M5,M9:M12)=0,"",SUM(M4:M5))</f>
         <v>2.91</v>
       </c>
       <c r="N6" s="15" t="str">
-        <f>IF(COUNT(N2:N3,N4:N5,N9:N10)=0,"",SUM(N4:N5))</f>
+        <f>IF(COUNT(N2:N3,N4:N5,N9:N12)=0,"",SUM(N4:N5))</f>
         <v/>
       </c>
       <c r="O6" s="15" t="str">
-        <f>IF(COUNT(O2:O3,O4:O5,O9:O10)=0,"",SUM(O4:O5))</f>
+        <f>IF(COUNT(O2:O3,O4:O5,O9:O12)=0,"",SUM(O4:O5))</f>
         <v/>
       </c>
       <c r="P6" s="15" t="str">
-        <f>IF(COUNT(P2:P3,P4:P5,P9:P10)=0,"",SUM(P4:P5))</f>
+        <f>IF(COUNT(P2:P3,P4:P5,P9:P12)=0,"",SUM(P4:P5))</f>
         <v/>
       </c>
       <c r="Q6" s="15" t="str">
-        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q10)=0,"",SUM(Q4:Q5))</f>
+        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q12)=0,"",SUM(Q4:Q5))</f>
         <v/>
       </c>
       <c r="R6" s="15" t="str">
-        <f>IF(COUNT(R2:R3,R4:R5,R9:R10)=0,"",SUM(R4:R5))</f>
+        <f>IF(COUNT(R2:R3,R4:R5,R9:R12)=0,"",SUM(R4:R5))</f>
         <v/>
       </c>
     </row>
@@ -2958,67 +2958,67 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>IF(COUNT(C2:C3,C4:C5,C9:C10)=0,"",SUM(C2:C3)-C6)</f>
+        <f>IF(COUNT(C2:C3,C4:C5,C9:C12)=0,"",SUM(C2:C3)-C6)</f>
         <v>3.09</v>
       </c>
       <c r="D7" s="15">
-        <f>IF(COUNT(D2:D3,D4:D5,D9:D10)=0,"",SUM(D2:D3)-D6)</f>
+        <f>IF(COUNT(D2:D3,D4:D5,D9:D12)=0,"",SUM(D2:D3)-D6)</f>
         <v>7.28</v>
       </c>
       <c r="E7" s="15">
-        <f>IF(COUNT(E2:E3,E4:E5,E9:E10)=0,"",SUM(E2:E3)-E6)</f>
+        <f>IF(COUNT(E2:E3,E4:E5,E9:E12)=0,"",SUM(E2:E3)-E6)</f>
         <v>7.58</v>
       </c>
       <c r="F7" s="15">
-        <f>IF(COUNT(F2:F3,F4:F5,F9:F10)=0,"",SUM(F2:F3)-F6)</f>
+        <f>IF(COUNT(F2:F3,F4:F5,F9:F12)=0,"",SUM(F2:F3)-F6)</f>
         <v>2.88</v>
       </c>
       <c r="G7" s="15">
-        <f>IF(COUNT(G2:G3,G4:G5,G9:G10)=0,"",SUM(G2:G3)-G6)</f>
+        <f>IF(COUNT(G2:G3,G4:G5,G9:G12)=0,"",SUM(G2:G3)-G6)</f>
         <v>3.12</v>
       </c>
       <c r="H7" s="15">
-        <f>IF(COUNT(H2:H3,H4:H5,H9:H10)=0,"",SUM(H2:H3)-H6)</f>
+        <f>IF(COUNT(H2:H3,H4:H5,H9:H12)=0,"",SUM(H2:H3)-H6)</f>
         <v>7.38</v>
       </c>
       <c r="I7" s="15">
-        <f>IF(COUNT(I2:I3,I4:I5,I9:I10)=0,"",SUM(I2:I3)-I6)</f>
+        <f>IF(COUNT(I2:I3,I4:I5,I9:I12)=0,"",SUM(I2:I3)-I6)</f>
         <v>7.74</v>
       </c>
       <c r="J7" s="15">
-        <f>IF(COUNT(J2:J3,J4:J5,J9:J10)=0,"",SUM(J2:J3)-J6)</f>
+        <f>IF(COUNT(J2:J3,J4:J5,J9:J12)=0,"",SUM(J2:J3)-J6)</f>
         <v>3.38</v>
       </c>
       <c r="K7" s="15">
-        <f>IF(COUNT(K2:K3,K4:K5,K9:K10)=0,"",SUM(K2:K3)-K6)</f>
+        <f>IF(COUNT(K2:K3,K4:K5,K9:K12)=0,"",SUM(K2:K3)-K6)</f>
         <v>3.44</v>
       </c>
       <c r="L7" s="15">
-        <f>IF(COUNT(L2:L3,L4:L5,L9:L10)=0,"",SUM(L2:L3)-L6)</f>
+        <f>IF(COUNT(L2:L3,L4:L5,L9:L12)=0,"",SUM(L2:L3)-L6)</f>
         <v>7.78</v>
       </c>
       <c r="M7" s="15">
-        <f>IF(COUNT(M2:M3,M4:M5,M9:M10)=0,"",SUM(M2:M3)-M6)</f>
+        <f>IF(COUNT(M2:M3,M4:M5,M9:M12)=0,"",SUM(M2:M3)-M6)</f>
         <v>8.03</v>
       </c>
       <c r="N7" s="15" t="str">
-        <f>IF(COUNT(N2:N3,N4:N5,N9:N10)=0,"",SUM(N2:N3)-N6)</f>
+        <f>IF(COUNT(N2:N3,N4:N5,N9:N12)=0,"",SUM(N2:N3)-N6)</f>
         <v/>
       </c>
       <c r="O7" s="15" t="str">
-        <f>IF(COUNT(O2:O3,O4:O5,O9:O10)=0,"",SUM(O2:O3)-O6)</f>
+        <f>IF(COUNT(O2:O3,O4:O5,O9:O12)=0,"",SUM(O2:O3)-O6)</f>
         <v/>
       </c>
       <c r="P7" s="15" t="str">
-        <f>IF(COUNT(P2:P3,P4:P5,P9:P10)=0,"",SUM(P2:P3)-P6)</f>
+        <f>IF(COUNT(P2:P3,P4:P5,P9:P12)=0,"",SUM(P2:P3)-P6)</f>
         <v/>
       </c>
       <c r="Q7" s="15" t="str">
-        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q10)=0,"",SUM(Q2:Q3)-Q6)</f>
+        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q12)=0,"",SUM(Q2:Q3)-Q6)</f>
         <v/>
       </c>
       <c r="R7" s="15" t="str">
-        <f>IF(COUNT(R2:R3,R4:R5,R9:R10)=0,"",SUM(R2:R3)-R6)</f>
+        <f>IF(COUNT(R2:R3,R4:R5,R9:R12)=0,"",SUM(R2:R3)-R6)</f>
         <v/>
       </c>
     </row>
@@ -3124,231 +3124,331 @@
       <c r="R10" s="10"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total debt service costs</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Calculated</t>
-        </is>
-      </c>
-      <c r="C11" s="15">
-        <f>IF(COUNT(C2:C3,C4:C5,C9:C10)=0,"",SUM(C9:C10))</f>
-        <v>4.35</v>
-      </c>
-      <c r="D11" s="15">
-        <f>IF(COUNT(D2:D3,D4:D5,D9:D10)=0,"",SUM(D9:D10))</f>
-        <v>4.33</v>
-      </c>
-      <c r="E11" s="15">
-        <f>IF(COUNT(E2:E3,E4:E5,E9:E10)=0,"",SUM(E9:E10))</f>
-        <v>4.32</v>
-      </c>
-      <c r="F11" s="15">
-        <f>IF(COUNT(F2:F3,F4:F5,F9:F10)=0,"",SUM(F9:F10))</f>
-        <v>4.31</v>
-      </c>
-      <c r="G11" s="15">
-        <f>IF(COUNT(G2:G3,G4:G5,G9:G10)=0,"",SUM(G9:G10))</f>
-        <v>4.28</v>
-      </c>
-      <c r="H11" s="15">
-        <f>IF(COUNT(H2:H3,H4:H5,H9:H10)=0,"",SUM(H9:H10))</f>
-        <v>4.29</v>
-      </c>
-      <c r="I11" s="15">
-        <f>IF(COUNT(I2:I3,I4:I5,I9:I10)=0,"",SUM(I9:I10))</f>
-        <v>4.27</v>
-      </c>
-      <c r="J11" s="15">
-        <f>IF(COUNT(J2:J3,J4:J5,J9:J10)=0,"",SUM(J9:J10))</f>
-        <v>4.27</v>
-      </c>
-      <c r="K11" s="15">
-        <f>IF(COUNT(K2:K3,K4:K5,K9:K10)=0,"",SUM(K9:K10))</f>
-        <v>4.27</v>
-      </c>
-      <c r="L11" s="15">
-        <f>IF(COUNT(L2:L3,L4:L5,L9:L10)=0,"",SUM(L9:L10))</f>
-        <v>4.28</v>
-      </c>
-      <c r="M11" s="15">
-        <f>IF(COUNT(M2:M3,M4:M5,M9:M10)=0,"",SUM(M9:M10))</f>
-        <v>4.29</v>
-      </c>
-      <c r="N11" s="15" t="str">
-        <f>IF(COUNT(N2:N3,N4:N5,N9:N10)=0,"",SUM(N9:N10))</f>
-        <v/>
-      </c>
-      <c r="O11" s="15" t="str">
-        <f>IF(COUNT(O2:O3,O4:O5,O9:O10)=0,"",SUM(O9:O10))</f>
-        <v/>
-      </c>
-      <c r="P11" s="15" t="str">
-        <f>IF(COUNT(P2:P3,P4:P5,P9:P10)=0,"",SUM(P9:P10))</f>
-        <v/>
-      </c>
-      <c r="Q11" s="15" t="str">
-        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q10)=0,"",SUM(Q9:Q10))</f>
-        <v/>
-      </c>
-      <c r="R11" s="15" t="str">
-        <f>IF(COUNT(R2:R3,R4:R5,R9:R10)=0,"",SUM(R9:R10))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12"/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interest rate swap settlements</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service</t>
+        </is>
+      </c>
+      <c r="C11" s="10">
+        <v>0.06</v>
+      </c>
+      <c r="D11" s="10">
+        <v>0.05</v>
+      </c>
+      <c r="E11" s="10">
+        <v>0.04</v>
+      </c>
+      <c r="F11" s="10">
+        <v>0.03</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="H11" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="I11" s="10">
+        <v>-0.01</v>
+      </c>
+      <c r="J11" s="10">
+        <v>-0.02</v>
+      </c>
+      <c r="K11" s="10">
+        <v>-0.03</v>
+      </c>
+      <c r="L11" s="10">
+        <v>-0.02</v>
+      </c>
+      <c r="M11" s="10">
+        <v>-0.03</v>
+      </c>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Agency fees</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service</t>
+        </is>
+      </c>
+      <c r="C12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="D12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="F12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="G12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="H12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="I12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="J12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="K12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="L12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="M12" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+    </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">Total debt service costs</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated</t>
+        </is>
+      </c>
+      <c r="C13" s="15">
+        <f>IF(COUNT(C2:C3,C4:C5,C9:C12)=0,"",SUM(C9:C12))</f>
+        <v>4.43</v>
+      </c>
+      <c r="D13" s="15">
+        <f>IF(COUNT(D2:D3,D4:D5,D9:D12)=0,"",SUM(D9:D12))</f>
+        <v>4.4</v>
+      </c>
+      <c r="E13" s="15">
+        <f>IF(COUNT(E2:E3,E4:E5,E9:E12)=0,"",SUM(E9:E12))</f>
+        <v>4.38</v>
+      </c>
+      <c r="F13" s="15">
+        <f>IF(COUNT(F2:F3,F4:F5,F9:F12)=0,"",SUM(F9:F12))</f>
+        <v>4.36</v>
+      </c>
+      <c r="G13" s="15">
+        <f>IF(COUNT(G2:G3,G4:G5,G9:G12)=0,"",SUM(G9:G12))</f>
+        <v>4.32</v>
+      </c>
+      <c r="H13" s="15">
+        <f>IF(COUNT(H2:H3,H4:H5,H9:H12)=0,"",SUM(H9:H12))</f>
+        <v>4.32</v>
+      </c>
+      <c r="I13" s="15">
+        <f>IF(COUNT(I2:I3,I4:I5,I9:I12)=0,"",SUM(I9:I12))</f>
+        <v>4.28</v>
+      </c>
+      <c r="J13" s="15">
+        <f>IF(COUNT(J2:J3,J4:J5,J9:J12)=0,"",SUM(J9:J12))</f>
+        <v>4.27</v>
+      </c>
+      <c r="K13" s="15">
+        <f>IF(COUNT(K2:K3,K4:K5,K9:K12)=0,"",SUM(K9:K12))</f>
+        <v>4.26</v>
+      </c>
+      <c r="L13" s="15">
+        <f>IF(COUNT(L2:L3,L4:L5,L9:L12)=0,"",SUM(L9:L12))</f>
+        <v>4.28</v>
+      </c>
+      <c r="M13" s="15">
+        <f>IF(COUNT(M2:M3,M4:M5,M9:M12)=0,"",SUM(M9:M12))</f>
+        <v>4.28</v>
+      </c>
+      <c r="N13" s="15" t="str">
+        <f>IF(COUNT(N2:N3,N4:N5,N9:N12)=0,"",SUM(N9:N12))</f>
+        <v/>
+      </c>
+      <c r="O13" s="15" t="str">
+        <f>IF(COUNT(O2:O3,O4:O5,O9:O12)=0,"",SUM(O9:O12))</f>
+        <v/>
+      </c>
+      <c r="P13" s="15" t="str">
+        <f>IF(COUNT(P2:P3,P4:P5,P9:P12)=0,"",SUM(P9:P12))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="15" t="str">
+        <f>IF(COUNT(Q2:Q3,Q4:Q5,Q9:Q12)=0,"",SUM(Q9:Q12))</f>
+        <v/>
+      </c>
+      <c r="R13" s="15" t="str">
+        <f>IF(COUNT(R2:R3,R4:R5,R9:R12)=0,"",SUM(R9:R12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR - quarter</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C13" s="16">
-        <f>IFERROR(C7/C11,"")</f>
-        <v>0.710345</v>
-      </c>
-      <c r="D13" s="16">
-        <f>IFERROR(D7/D11,"")</f>
-        <v>1.681293</v>
-      </c>
-      <c r="E13" s="16">
-        <f>IFERROR(E7/E11,"")</f>
-        <v>1.75463</v>
-      </c>
-      <c r="F13" s="16">
-        <f>IFERROR(F7/F11,"")</f>
-        <v>0.668213</v>
-      </c>
-      <c r="G13" s="16">
-        <f>IFERROR(G7/G11,"")</f>
-        <v>0.728972</v>
-      </c>
-      <c r="H13" s="16">
-        <f>IFERROR(H7/H11,"")</f>
-        <v>1.72028</v>
-      </c>
-      <c r="I13" s="16">
-        <f>IFERROR(I7/I11,"")</f>
-        <v>1.812646</v>
-      </c>
-      <c r="J13" s="16">
-        <f>IFERROR(J7/J11,"")</f>
+      <c r="C15" s="16">
+        <f>IFERROR(C7/C13,"")</f>
+        <v>0.697517</v>
+      </c>
+      <c r="D15" s="16">
+        <f>IFERROR(D7/D13,"")</f>
+        <v>1.654545</v>
+      </c>
+      <c r="E15" s="16">
+        <f>IFERROR(E7/E13,"")</f>
+        <v>1.730594</v>
+      </c>
+      <c r="F15" s="16">
+        <f>IFERROR(F7/F13,"")</f>
+        <v>0.66055</v>
+      </c>
+      <c r="G15" s="16">
+        <f>IFERROR(G7/G13,"")</f>
+        <v>0.722222</v>
+      </c>
+      <c r="H15" s="16">
+        <f>IFERROR(H7/H13,"")</f>
+        <v>1.708333</v>
+      </c>
+      <c r="I15" s="16">
+        <f>IFERROR(I7/I13,"")</f>
+        <v>1.808411</v>
+      </c>
+      <c r="J15" s="16">
+        <f>IFERROR(J7/J13,"")</f>
         <v>0.791569</v>
       </c>
-      <c r="K13" s="16">
-        <f>IFERROR(K7/K11,"")</f>
-        <v>0.805621</v>
-      </c>
-      <c r="L13" s="16">
-        <f>IFERROR(L7/L11,"")</f>
+      <c r="K15" s="16">
+        <f>IFERROR(K7/K13,"")</f>
+        <v>0.807512</v>
+      </c>
+      <c r="L15" s="16">
+        <f>IFERROR(L7/L13,"")</f>
         <v>1.817757</v>
       </c>
-      <c r="M13" s="16">
-        <f>IFERROR(M7/M11,"")</f>
-        <v>1.871795</v>
-      </c>
-      <c r="N13" s="16" t="str">
-        <f>IFERROR(N7/N11,"")</f>
-        <v/>
-      </c>
-      <c r="O13" s="16" t="str">
-        <f>IFERROR(O7/O11,"")</f>
-        <v/>
-      </c>
-      <c r="P13" s="16" t="str">
-        <f>IFERROR(P7/P11,"")</f>
-        <v/>
-      </c>
-      <c r="Q13" s="16" t="str">
-        <f>IFERROR(Q7/Q11,"")</f>
-        <v/>
-      </c>
-      <c r="R13" s="16" t="str">
-        <f>IFERROR(R7/R11,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="M15" s="16">
+        <f>IFERROR(M7/M13,"")</f>
+        <v>1.876168</v>
+      </c>
+      <c r="N15" s="16" t="str">
+        <f>IFERROR(N7/N13,"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="16" t="str">
+        <f>IFERROR(O7/O13,"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="16" t="str">
+        <f>IFERROR(P7/P13,"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="16" t="str">
+        <f>IFERROR(Q7/Q13,"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="16" t="str">
+        <f>IFERROR(R7/R13,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">DSCR - LTM</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Calculated</t>
         </is>
       </c>
-      <c r="C14" s="16" t="str">
+      <c r="C16" s="16" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="D14" s="16" t="str">
+      <c r="D16" s="16" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="E14" s="16" t="str">
+      <c r="E16" s="16" t="str">
         <f>""</f>
         <v/>
       </c>
-      <c r="F14" s="16">
-        <f>IF(COUNT(C7:F7)&lt;4,"",IFERROR(SUM(C7:F7)/SUM(C11:F11),""))</f>
-        <v>1.203351</v>
-      </c>
-      <c r="G14" s="16">
-        <f>IF(COUNT(D7:G7)&lt;4,"",IFERROR(SUM(D7:G7)/SUM(D11:G11),""))</f>
-        <v>1.209977</v>
-      </c>
-      <c r="H14" s="16">
-        <f>IF(COUNT(E7:H7)&lt;4,"",IFERROR(SUM(E7:H7)/SUM(E11:H11),""))</f>
-        <v>1.218605</v>
-      </c>
-      <c r="I14" s="16">
-        <f>IF(COUNT(F7:I7)&lt;4,"",IFERROR(SUM(F7:I7)/SUM(F11:I11),""))</f>
-        <v>1.231487</v>
-      </c>
-      <c r="J14" s="16">
-        <f>IF(COUNT(G7:J7)&lt;4,"",IFERROR(SUM(G7:J7)/SUM(G11:J11),""))</f>
-        <v>1.263589</v>
-      </c>
-      <c r="K14" s="16">
-        <f>IF(COUNT(H7:K7)&lt;4,"",IFERROR(SUM(H7:K7)/SUM(H11:K11),""))</f>
-        <v>1.283041</v>
-      </c>
-      <c r="L14" s="16">
-        <f>IF(COUNT(I7:L7)&lt;4,"",IFERROR(SUM(I7:L7)/SUM(I11:L11),""))</f>
+      <c r="F16" s="16">
+        <f>IF(COUNT(C7:F7)&lt;4,"",IFERROR(SUM(C7:F7)/SUM(C13:F13),""))</f>
+        <v>1.185544</v>
+      </c>
+      <c r="G16" s="16">
+        <f>IF(COUNT(D7:G7)&lt;4,"",IFERROR(SUM(D7:G7)/SUM(D13:G13),""))</f>
+        <v>1.194731</v>
+      </c>
+      <c r="H16" s="16">
+        <f>IF(COUNT(E7:H7)&lt;4,"",IFERROR(SUM(E7:H7)/SUM(E13:H13),""))</f>
+        <v>1.205984</v>
+      </c>
+      <c r="I16" s="16">
+        <f>IF(COUNT(F7:I7)&lt;4,"",IFERROR(SUM(F7:I7)/SUM(F13:I13),""))</f>
+        <v>1.222222</v>
+      </c>
+      <c r="J16" s="16">
+        <f>IF(COUNT(G7:J7)&lt;4,"",IFERROR(SUM(G7:J7)/SUM(G13:J13),""))</f>
+        <v>1.257708</v>
+      </c>
+      <c r="K16" s="16">
+        <f>IF(COUNT(H7:K7)&lt;4,"",IFERROR(SUM(H7:K7)/SUM(H13:K13),""))</f>
+        <v>1.280794</v>
+      </c>
+      <c r="L16" s="16">
+        <f>IF(COUNT(I7:L7)&lt;4,"",IFERROR(SUM(I7:L7)/SUM(I13:L13),""))</f>
         <v>1.307197</v>
       </c>
-      <c r="M14" s="16">
-        <f>IF(COUNT(J7:M7)&lt;4,"",IFERROR(SUM(J7:M7)/SUM(J11:M11),""))</f>
-        <v>1.322618</v>
-      </c>
-      <c r="N14" s="16" t="str">
-        <f>IF(COUNT(K7:N7)&lt;4,"",IFERROR(SUM(K7:N7)/SUM(K11:N11),""))</f>
-        <v/>
-      </c>
-      <c r="O14" s="16" t="str">
-        <f>IF(COUNT(L7:O7)&lt;4,"",IFERROR(SUM(L7:O7)/SUM(L11:O11),""))</f>
-        <v/>
-      </c>
-      <c r="P14" s="16" t="str">
-        <f>IF(COUNT(M7:P7)&lt;4,"",IFERROR(SUM(M7:P7)/SUM(M11:P11),""))</f>
-        <v/>
-      </c>
-      <c r="Q14" s="16" t="str">
-        <f>IF(COUNT(N7:Q7)&lt;4,"",IFERROR(SUM(N7:Q7)/SUM(N11:Q11),""))</f>
-        <v/>
-      </c>
-      <c r="R14" s="16" t="str">
-        <f>IF(COUNT(O7:R7)&lt;4,"",IFERROR(SUM(O7:R7)/SUM(O11:R11),""))</f>
+      <c r="M16" s="16">
+        <f>IF(COUNT(J7:M7)&lt;4,"",IFERROR(SUM(J7:M7)/SUM(J13:M13),""))</f>
+        <v>1.324166</v>
+      </c>
+      <c r="N16" s="16" t="str">
+        <f>IF(COUNT(K7:N7)&lt;4,"",IFERROR(SUM(K7:N7)/SUM(K13:N13),""))</f>
+        <v/>
+      </c>
+      <c r="O16" s="16" t="str">
+        <f>IF(COUNT(L7:O7)&lt;4,"",IFERROR(SUM(L7:O7)/SUM(L13:O13),""))</f>
+        <v/>
+      </c>
+      <c r="P16" s="16" t="str">
+        <f>IF(COUNT(M7:P7)&lt;4,"",IFERROR(SUM(M7:P7)/SUM(M13:P13),""))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="16" t="str">
+        <f>IF(COUNT(N7:Q7)&lt;4,"",IFERROR(SUM(N7:Q7)/SUM(N13:Q13),""))</f>
+        <v/>
+      </c>
+      <c r="R16" s="16" t="str">
+        <f>IF(COUNT(O7:R7)&lt;4,"",IFERROR(SUM(O7:R7)/SUM(O13:R13),""))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard builder: Charts tab values all display with 1 decimal
Every value cell on the example workbooks' Charts tab now uses the 0.0
number format (full precision is kept in the cell).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -1903,34 +1903,34 @@
       <c r="D4" s="8">
         <v>1</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="9">
         <v>1.62</v>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <v>1.84</v>
       </c>
-      <c r="G4" s="10">
+      <c r="G4" s="9">
         <v>2.57</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="9">
         <v>3.03</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="9">
         <v>3.41</v>
       </c>
-      <c r="J4" s="10">
+      <c r="J4" s="9">
         <v>4.12</v>
       </c>
-      <c r="K4" s="10">
+      <c r="K4" s="9">
         <v>3.46</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="9">
         <v>3.92</v>
       </c>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1995,34 +1995,34 @@
       <c r="D6" s="8">
         <v>1</v>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <v>-0.41</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <v>0.12</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <v>0.88</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="9">
         <v>1.31</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="9">
         <v>1.69</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="9">
         <v>2.27</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="9">
         <v>1.66</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="9">
         <v>2.07</v>
       </c>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Dashboard builder: same Side Table layout in both example workbooks
Bluefield's Side Table now matches Ridgeline's (Item / Balance / MoM with
cash, reserves and debt rows) instead of an empty Item / Value header.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -2594,7 +2594,97 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Balance</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MoM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unrestricted cash</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$1.2MM</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-$0.3MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O&amp;M reserve</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$1.85MM</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+$0.05MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debt service reserve</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$8.62MM</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flat</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Term loan</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$96.4MM</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-$0.9MM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Revolver</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$0.0MM</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flat</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard builder: YTD section on monthly charts, DSCR quarter axis, YTD-first table
- Page 1 charts gain a YTD section at the right (Jan..Current month for
  both years, stacked where the chart is), on its own scale behind a
  divider so year-to-date totals do not flatten the monthly bars.
  Charts tab gets an optional YTD Method column after Dec (Sum default,
  Average, None); the month columns the Table formulas read are unmoved.
- Page 2's LTM DSCR panel gets its own quarter axis; quarter labels fall
  back to the short form (Q3 24) when the full label would not fit.
- The comparison table shows YTD columns first, then the month; the
  example titles read "YTD & Monthly" and older "Monthly & YTD" titles
  are flipped to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AJKVLHooDq3QqacfYhYJhs
</commit_message>
<xml_diff>
--- a/dashboard-builder/Bluefield-Example-Inputs.xlsx
+++ b/dashboard-builder/Bluefield-Example-Inputs.xlsx
@@ -258,209 +258,223 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Every chart shows the Prior year and Current year from Settings side by side, month by month.</t>
+          <t xml:space="preserve">               Every chart shows the Prior year and Current year from Settings side by side, month by month,</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Enter full precision here (e.g. 3.92); the Decimals column only controls how the chart labels are rounded.</t>
+          <t xml:space="preserve">               plus a YTD section on the right (Jan through Current month, both years).  "YTD Method": Sum (default),</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Footnotes  -  explain a month on a chart.  Pick the chart from the dropdown, or leave "Chart" blank to mark that month on every chart.</t>
+          <t xml:space="preserve">               Average (for percentages), or None to leave the YTD section off that chart.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">               The month label gets a small number and the note prints under the charts.</t>
+          <t xml:space="preserve">               Enter full precision here (e.g. 3.92); the Decimals column only controls how the chart labels are rounded.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Table  -  any number of rows.  The variance is calculated for you; "Better When" sets whether it shows green or red.</t>
+          <t xml:space="preserve">Footnotes  -  explain a month on a chart.  Pick the chart from the dropdown, or leave "Chart" blank to mark that month on every chart.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Month Actual and YTD Actual (black cells) are formulas: rows with a "From Chart" sum that chart on the Charts tab for the</t>
+          <t xml:space="preserve">               The month label gets a small number and the note prints under the charts.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Current year, for the Current month and Jan through it (add a "From Component" to use one component, e.g. Contracted).</t>
+          <t xml:space="preserve">Table  -  any number of rows.  The variance is calculated for you; "Better When" sets whether it shows green or red.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">               O&amp;M expense defaults to Revenue - Operating income.  Type a number over any formula to override it; the PDF uses the cell value.</t>
+          <t xml:space="preserve">               Month Actual and YTD Actual (black cells) are formulas: rows with a "From Chart" sum that chart on the Charts tab for the</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Rows with no "From Chart" and no formula: type the actuals yourself.</t>
+          <t xml:space="preserve">               Current year, for the Current month and Jan through it (add a "From Component" to use one component, e.g. Contracted).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">               "EV Basis": if the EV Case values were pro-rated from quarterly, semi-annual or annual figures, pick that here.  The EV Case</t>
+          <t xml:space="preserve">               O&amp;M expense defaults to Revenue - Operating income.  Type a number over any formula to override it; the PDF uses the cell value.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">               values get a small letter (a, b, ...) and a footnote under the table explains it.  Monthly (the default) adds nothing.</t>
+          <t xml:space="preserve">               Rows with no "From Chart" and no formula: type the actuals yourself.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
+          <t xml:space="preserve">               "EV Basis": if the EV Case values were pro-rated from quarterly, semi-annual or annual figures, pick that here.  The EV Case</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
+          <t xml:space="preserve">               values get a small letter (a, b, ...) and a footnote under the table explains it.  Monthly (the default) adds nothing.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
+          <t xml:space="preserve">               "YTD Method": Sum (default) adds the months up; Average averages them (use for percentages like capacity factor).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
+          <t xml:space="preserve">               Month EV Case and YTD EV Case are always typed in.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Service  -  a running quarterly history for page 2: one column per quarter (Q1 2024 to Q4 2027).  Fill in each quarter when it closes;</t>
+          <t xml:space="preserve">Commentary  -  Heading + Text pairs for the bottom-right box.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">               nothing ever needs shifting.  Page 2 shows the last completed quarter before the Current month's quarter and the 3 before it</t>
+          <t xml:space="preserve">Side Table  -  a free-form grid for the bottom-right box.  Row 1 = column headers.  Values print exactly as they appear in Excel.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">               (Current month Aug -&gt; through Q2; Dec -&gt; through Q3).  Add more quarters by adding columns with labels like "Q1 2028".</t>
+          <t xml:space="preserve">Debt Service  -  a running quarterly history for page 2: one column per quarter (Q1 2024 to Q4 2027).  Fill in each quarter when it closes;</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">               Role: Revenue, Expense or Debt service.  Enter expenses and debt service as positive numbers.  The black "Calculated</t>
+          <t xml:space="preserve">               nothing ever needs shifting.  Page 2 shows the last completed quarter before the Current month's quarter and the 3 before it</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">               rows do the math: Total O&amp;M costs, CFADS = Revenue - Total O&amp;M costs, Total debt service costs, DSCR, and DSCR - LTM</t>
+          <t xml:space="preserve">               (Current month Aug -&gt; through Q2; Dec -&gt; through Q3).  Add more quarters by adding columns with labels like "Q1 2028".</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">               (last 4 quarters of CFADS / last 4 quarters of debt service).  To add a line (e.g. LC fees), insert the row between two</t>
+          <t xml:space="preserve">               Role: Revenue, Expense or Debt service.  Enter expenses and debt service as positive numbers.  The black "Calculated</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">               rows of the same block so the totals' ranges grow to include it.  The PDF recalculates from the input rows.</t>
+          <t xml:space="preserve">               rows do the math: Total O&amp;M costs, CFADS = Revenue - Total O&amp;M costs, Total debt service costs, DSCR, and DSCR - LTM</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+          <t xml:space="preserve">               (last 4 quarters of CFADS / last 4 quarters of debt service).  To add a line (e.g. LC fees), insert the row between two</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+          <t xml:space="preserve">               rows of the same block so the totals' ranges grow to include it.  The PDF recalculates from the input rows.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t xml:space="preserve">Reserves  -  one row per reserve account (DSR, O&amp;M reserve, ...): Required balance and Balance available.  Shown on page 2 below the DSCR chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">               with the % funded; anything under 100% is flagged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t xml:space="preserve">DSCR Notes  -  optional Heading + Text pairs shown on page 2 below the reserves.</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">Tips</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+          <t xml:space="preserve">-  Do not rename the tabs or the column headers in row 1.  You can add, delete or reorder rows freely.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  Copy this workbook for each asset (one workbook = one dashboard).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-  The Chart dropdowns list the names on the Charts tab automatically (from a hidden "Lists" tab).  Add a chart there and it appears in the dropdowns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t xml:space="preserve">-  Your data never leaves your computer: the builder page reads the file locally in the browser.</t>
         </is>
@@ -1339,7 +1353,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operating and Financial Performance vs. EV Case - Monthly &amp; YTD</t>
+          <t xml:space="preserve">Operating and Financial Performance vs. EV Case - YTD &amp; Monthly</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1714,6 +1728,7 @@
     <col min="14" max="14" width="8" customWidth="1"/>
     <col min="15" max="15" width="8" customWidth="1"/>
     <col min="16" max="16" width="8" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1797,6 +1812,11 @@
           <t xml:space="preserve">Dec</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YTD Method</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -1839,6 +1859,11 @@
       <c r="N2" s="9"/>
       <c r="O2" s="9"/>
       <c r="P2" s="9"/>
+      <c r="Q2" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1888,6 +1913,11 @@
       </c>
       <c r="P3" s="9">
         <v>21.8</v>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -1931,6 +1961,11 @@
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
       <c r="P4" s="9"/>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1980,6 +2015,11 @@
       </c>
       <c r="P5" s="9">
         <v>1.4</v>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2023,6 +2063,11 @@
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -2073,8 +2118,18 @@
       <c r="P7" s="9">
         <v>-0.5</v>
       </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sum</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q500">
+      <formula1>"Sum,Average,None"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>